<commit_message>
Fixed name of the sheet
</commit_message>
<xml_diff>
--- a/Project-5-AdventureWorks-Sales-Performance-Analysis/excel/01_eda/01_decline_profit.xlsx
+++ b/Project-5-AdventureWorks-Sales-Performance-Analysis/excel/01_eda/01_decline_profit.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="RawData" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="All_Data" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -139,7 +139,7 @@
     <numFmt numFmtId="165" formatCode="0"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -161,6 +161,13 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -179,7 +186,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
+  <cellStyleXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -203,6 +210,24 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -230,14 +255,29 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="12">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="Pivot Table Field" xfId="20"/>
+    <cellStyle name="Pivot Table Corner" xfId="21"/>
+    <cellStyle name="Pivot Table Value" xfId="22"/>
+    <cellStyle name="Pivot Table Category" xfId="23"/>
+    <cellStyle name="Pivot Table Title" xfId="24"/>
+    <cellStyle name="Pivot Table Result" xfId="25"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -356,13 +396,15 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="3" style="2" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="13.4"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="3" width="16.74"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="12" min="7" style="2" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="2" width="12.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="3" width="15.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="4" width="13.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="4" width="13.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="13.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="24" style="0" width="16.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="10.2"/>
   </cols>

</xml_diff>

<commit_message>
Changed the pivot tables formula
</commit_message>
<xml_diff>
--- a/Project-5-AdventureWorks-Sales-Performance-Analysis/excel/01_eda/01_decline_profit.xlsx
+++ b/Project-5-AdventureWorks-Sales-Performance-Analysis/excel/01_eda/01_decline_profit.xlsx
@@ -5,19 +5,15 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="All_Data" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Clean_Data" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Pivot Table_Clean_Data_1" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Pivot Table_All_Data_1" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">All_Data!$A$1:$Z$15</definedName>
-  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId7"/>
+    <pivotCache cacheId="1" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -28,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="48">
   <si>
     <t xml:space="preserve">year</t>
   </si>
@@ -144,18 +140,6 @@
     <t xml:space="preserve">Data</t>
   </si>
   <si>
-    <t xml:space="preserve">Total Sum - total_qty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Sum - net_profit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Average - gross_margin_pct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Average - profit_yoy_pct</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sum - total_qty</t>
   </si>
   <si>
@@ -166,6 +150,21 @@
   </si>
   <si>
     <t xml:space="preserve">Average - profit_yoy_pct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Min - decline_rank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average - returns_per_qty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sum - profit_yoy_pct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sum - qty_yoy_pct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sum - profit_delta</t>
   </si>
   <si>
     <t xml:space="preserve">Total Result</t>
@@ -219,7 +218,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="19">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -252,42 +251,14 @@
       <left/>
       <right/>
       <top style="medium"/>
-      <bottom/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right style="medium"/>
       <top style="medium"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="medium"/>
-      <right style="thin"/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="medium"/>
-      <top style="thin"/>
-      <bottom/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
@@ -312,14 +283,7 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
+      <left/>
       <right style="medium"/>
       <top/>
       <bottom style="thin"/>
@@ -348,16 +312,16 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left/>
-      <right style="thin"/>
+      <right style="medium"/>
       <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left/>
+      <left style="medium"/>
       <right style="thin"/>
       <top/>
-      <bottom style="thin"/>
+      <bottom/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
@@ -383,20 +347,6 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
       <right style="medium"/>
       <top style="thin"/>
       <bottom style="medium"/>
@@ -446,7 +396,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -499,7 +449,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -507,159 +457,83 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="20" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="24" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="9" xfId="24" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="11" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="12" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="14" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="8" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="8" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="15" xfId="24" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="13" xfId="24" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="14" xfId="24" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="15" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="16" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="17" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="18" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="25" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="25" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="25" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="8" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="23" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="8" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="9" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="11" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="12" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="12" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="19" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="25" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="13" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="23" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="13" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="14" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="20" xfId="24" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="21" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="22" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="22" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="23" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="24" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="24" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="24" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="25" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="16" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="17" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="17" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="17" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="18" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -690,14 +564,10 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" recordCount="8" createdVersion="3">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" recordCount="14" createdVersion="3">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:Z9" sheet="Clean_Data"/>
+    <worksheetSource ref="A1:Z15" sheet="All_Data"/>
   </cacheSource>
   <cacheFields count="26">
     <cacheField name="year" numFmtId="0">
@@ -707,7 +577,8 @@
       </sharedItems>
     </cacheField>
     <cacheField name="total_qty" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="5304" maxValue="45314" count="8">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="45314" count="9">
+        <n v="0"/>
         <n v="5304"/>
         <n v="5610"/>
         <n v="5689"/>
@@ -761,7 +632,8 @@
       </sharedItems>
     </cacheField>
     <cacheField name="net_profit" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="69126.99" maxValue="3690735.2" count="8">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0" maxValue="3690735.2" count="9">
+        <n v="0"/>
         <n v="69126.99"/>
         <n v="92660.11"/>
         <n v="250936.12"/>
@@ -872,29 +744,51 @@
       </sharedItems>
     </cacheField>
     <cacheField name="continent" numFmtId="0">
-      <sharedItems count="1">
+      <sharedItems count="4">
         <s v="0"/>
+        <s v="Europe"/>
+        <s v="North America"/>
+        <s v="Pacific"/>
       </sharedItems>
     </cacheField>
     <cacheField name="sales_qty" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="0" count="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="3496046" count="7">
         <n v="0"/>
+        <n v="864233"/>
+        <n v="1249024"/>
+        <n v="1353420"/>
+        <n v="1944835"/>
+        <n v="2218218"/>
+        <n v="3496046"/>
       </sharedItems>
     </cacheField>
     <cacheField name="net_sales_value" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="0" count="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0" maxValue="4270567.72329797" count="7">
         <n v="0"/>
+        <n v="34930.8751287839"/>
+        <n v="1781554.47393563"/>
+        <n v="3211651.83251283"/>
+        <n v="3218911.38403874"/>
+        <n v="3293496.74615632"/>
+        <n v="4270567.72329797"/>
       </sharedItems>
     </cacheField>
     <cacheField name="returns_per_qty" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="0" count="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0" maxValue="375.741416680663" count="7">
         <n v="0"/>
+        <n v="175.669374322156"/>
+        <n v="190.12575110637"/>
+        <n v="215.69839258202"/>
+        <n v="253.814111575181"/>
+        <n v="284.275128347168"/>
+        <n v="375.741416680663"/>
       </sharedItems>
     </cacheField>
     <cacheField name="source" numFmtId="0">
-      <sharedItems count="2">
+      <sharedItems count="3">
         <s v="Categories"/>
         <s v="Overall"/>
+        <s v="Territory"/>
       </sharedItems>
     </cacheField>
   </cacheFields>
@@ -902,17 +796,17 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" count="8">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" count="14">
   <r>
     <x v="0"/>
-    <x v="6"/>
+    <x v="7"/>
     <x v="2"/>
     <x v="2"/>
     <x v="2"/>
     <x v="1"/>
     <x v="1"/>
     <x v="1"/>
-    <x v="7"/>
+    <x v="8"/>
     <x v="0"/>
     <x v="0"/>
     <x v="0"/>
@@ -933,14 +827,14 @@
   </r>
   <r>
     <x v="1"/>
-    <x v="7"/>
+    <x v="8"/>
     <x v="1"/>
     <x v="1"/>
     <x v="1"/>
     <x v="2"/>
     <x v="2"/>
     <x v="2"/>
-    <x v="5"/>
+    <x v="6"/>
     <x v="1"/>
     <x v="1"/>
     <x v="1"/>
@@ -961,14 +855,14 @@
   </r>
   <r>
     <x v="0"/>
-    <x v="4"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="2"/>
+    <x v="5"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="3"/>
     <x v="0"/>
     <x v="0"/>
     <x v="0"/>
@@ -989,14 +883,14 @@
   </r>
   <r>
     <x v="1"/>
-    <x v="5"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="3"/>
+    <x v="6"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="4"/>
     <x v="0"/>
     <x v="0"/>
     <x v="0"/>
@@ -1017,14 +911,14 @@
   </r>
   <r>
     <x v="0"/>
-    <x v="1"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="6"/>
+    <x v="2"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="7"/>
     <x v="0"/>
     <x v="0"/>
     <x v="0"/>
@@ -1045,14 +939,14 @@
   </r>
   <r>
     <x v="1"/>
-    <x v="2"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="4"/>
+    <x v="3"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="5"/>
     <x v="0"/>
     <x v="0"/>
     <x v="0"/>
@@ -1073,14 +967,14 @@
   </r>
   <r>
     <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
     <x v="0"/>
     <x v="0"/>
     <x v="0"/>
@@ -1101,14 +995,14 @@
   </r>
   <r>
     <x v="1"/>
-    <x v="3"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="1"/>
+    <x v="4"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="2"/>
     <x v="0"/>
     <x v="0"/>
     <x v="0"/>
@@ -1127,12 +1021,180 @@
     <x v="0"/>
     <x v="0"/>
   </r>
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="3"/>
+    <x v="5"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="5"/>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="3"/>
+    <x v="2"/>
+    <x v="6"/>
+    <x v="6"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="3"/>
+    <x v="4"/>
+    <x v="3"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="6"/>
+    <x v="5"/>
+    <x v="1"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="3"/>
+    <x v="4"/>
+    <x v="1"/>
+    <x v="4"/>
+    <x v="2"/>
+  </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="DataPilot1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" showDrill="0" useAutoFormatting="0" itemPrintTitles="1" indent="0" outline="0" outlineData="0" compact="0" compactData="0">
-  <location ref="A5:U10" firstHeaderRow="1" firstDataRow="3" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
+  <location ref="A5:J9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
   <pivotFields count="26">
     <pivotField axis="axisRow" compact="0" showAll="0" defaultSubtotal="0" outline="0">
       <items count="2">
@@ -1150,10 +1212,10 @@
     <pivotField dataField="1" compact="0" showAll="0" outline="0"/>
     <pivotField compact="0" showAll="0"/>
     <pivotField compact="0" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
     <pivotField dataField="1" compact="0" showAll="0" outline="0"/>
     <pivotField dataField="1" compact="0" showAll="0" outline="0"/>
-    <pivotField axis="axisCol" compact="0" showAll="0" defaultSubtotal="0" outline="0">
+    <pivotField dataField="1" compact="0" showAll="0" outline="0"/>
+    <pivotField axis="axisPage" compact="0" showAll="0" defaultSubtotal="0" outline="0">
       <items count="4">
         <item x="0"/>
         <item x="1"/>
@@ -1165,30 +1227,24 @@
     <pivotField compact="0" showAll="0"/>
     <pivotField compact="0" showAll="0"/>
     <pivotField compact="0" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" showAll="0" outline="0"/>
+    <pivotField dataField="1" compact="0" showAll="0" outline="0"/>
     <pivotField axis="axisPage" compact="0" showAll="0" defaultSubtotal="0" outline="0">
-      <items count="7">
+      <items count="4">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisPage" compact="0" showAll="0" defaultSubtotal="0" outline="0">
-      <items count="1">
-        <item x="0"/>
       </items>
     </pivotField>
     <pivotField compact="0" showAll="0"/>
     <pivotField compact="0" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" showAll="0" outline="0"/>
     <pivotField axis="axisPage" compact="0" showAll="0" defaultSubtotal="0" outline="0">
-      <items count="2">
+      <items count="3">
         <item x="0"/>
         <item x="1"/>
+        <item x="2"/>
       </items>
     </pivotField>
   </pivotFields>
@@ -1206,82 +1262,29 @@
       <x v="2"/>
     </i>
   </rowItems>
-  <colFields count="2">
-    <field x="14"/>
+  <colFields count="1">
     <field x="-2"/>
   </colFields>
-  <colItems count="20">
-    <i>
+  <colItems count="1">
+    <i t="grand">
       <x v="0"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="14"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i>
-      <x v="18"/>
-    </i>
-    <i t="grand">
-      <x v="19"/>
     </i>
   </colItems>
   <pageFields count="3">
+    <pageField fld="14" hier="-1"/>
     <pageField fld="21" hier="-1"/>
     <pageField fld="25" hier="-1"/>
-    <pageField fld="20" hier="-1"/>
   </pageFields>
-  <dataFields count="4">
+  <dataFields count="9">
     <dataField name="Sum - total_qty" fld="1" subtotal="sum" numFmtId="165"/>
     <dataField name="Sum - net_profit" fld="8" subtotal="sum" numFmtId="167"/>
     <dataField name="Average - gross_margin_pct" fld="13" subtotal="average" numFmtId="166"/>
     <dataField name="Average - profit_yoy_pct" fld="12" subtotal="average" numFmtId="166"/>
+    <dataField name="Min - decline_rank" fld="20" subtotal="min" numFmtId="164"/>
+    <dataField name="Average - returns_per_qty" fld="24" subtotal="average" numFmtId="164"/>
+    <dataField name="Sum - profit_yoy_pct*" fld="12" subtotal="sum" numFmtId="166"/>
+    <dataField name="Sum - qty_yoy_pct" fld="11" subtotal="sum" numFmtId="166"/>
+    <dataField name="Sum - profit_delta" fld="19" subtotal="sum" numFmtId="164"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
 </pivotTableDefinition>
@@ -1395,7 +1398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="true">
+  <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Z50"/>
@@ -2135,7 +2138,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
         <v>2021</v>
       </c>
@@ -2215,7 +2218,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="n">
         <v>2021</v>
       </c>
@@ -2295,7 +2298,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
         <v>2021</v>
       </c>
@@ -2375,7 +2378,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="n">
         <v>2022</v>
       </c>
@@ -2455,7 +2458,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="n">
         <v>2022</v>
       </c>
@@ -2535,7 +2538,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="n">
         <v>2022</v>
       </c>
@@ -2622,19 +2625,6 @@
       <c r="B50" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z15">
-    <filterColumn colId="0">
-      <customFilters and="true">
-        <customFilter operator="**none**" val=""/>
-      </customFilters>
-    </filterColumn>
-    <filterColumn colId="25">
-      <filters>
-        <filter val="Categories"/>
-        <filter val="Overall"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2642,7 +2632,6 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2651,774 +2640,24 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z9"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="W1" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="X1" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z1" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B2" s="4" t="n">
-        <v>36230</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>9324203.79</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>5357119.66</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>3967084.13</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>770</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>276348.93</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>35460</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>3690735.2</v>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="2" t="n">
-        <v>42.55</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="P2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="W2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="X2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>45314</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>9185449.45</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>5296420.47</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>3889028.97</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>972</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>277297.17</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>44342</v>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>3611731.81</v>
-      </c>
-      <c r="J3" s="2" t="n">
-        <v>36230</v>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>3690735.2</v>
-      </c>
-      <c r="L3" s="2" t="n">
-        <v>25.07</v>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>-2.14</v>
-      </c>
-      <c r="N3" s="2" t="n">
-        <v>42.34</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="P3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="V3" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="W3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="X3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z3" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>25316</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>250936.12</v>
-      </c>
-      <c r="J4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="P4" s="3" t="n">
-        <v>399342.117799956</v>
-      </c>
-      <c r="Q4" s="3" t="n">
-        <v>148405.994799995</v>
-      </c>
-      <c r="R4" s="3" t="n">
-        <v>2.68812185758366</v>
-      </c>
-      <c r="S4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="V4" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="W4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="X4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>32493</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>318823.94</v>
-      </c>
-      <c r="J5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="P5" s="3" t="n">
-        <v>507330.989199908</v>
-      </c>
-      <c r="Q5" s="3" t="n">
-        <v>188507.051199988</v>
-      </c>
-      <c r="R5" s="3" t="n">
-        <v>2.68828158743257</v>
-      </c>
-      <c r="S5" s="3" t="n">
-        <v>7177</v>
-      </c>
-      <c r="T5" s="3" t="n">
-        <v>67887.8149999597</v>
-      </c>
-      <c r="U5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="V5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="W5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="X5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>5610</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>3647021.02</v>
-      </c>
-      <c r="J6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="P6" s="3" t="n">
-        <v>8768706.98490015</v>
-      </c>
-      <c r="Q6" s="3" t="n">
-        <v>5121685.96939992</v>
-      </c>
-      <c r="R6" s="3" t="n">
-        <v>1.70568672635527</v>
-      </c>
-      <c r="S6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U6" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="V6" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="W6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="X6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z6" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>5689</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>3477544.92</v>
-      </c>
-      <c r="J7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="P7" s="3" t="n">
-        <v>8468854.53000019</v>
-      </c>
-      <c r="Q7" s="3" t="n">
-        <v>4991309.60669985</v>
-      </c>
-      <c r="R7" s="3" t="n">
-        <v>1.6921437844365</v>
-      </c>
-      <c r="S7" s="3" t="n">
-        <v>79</v>
-      </c>
-      <c r="T7" s="3" t="n">
-        <v>-169476.092199898</v>
-      </c>
-      <c r="U7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="V7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="W7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="X7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z7" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>5304</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>69126.99</v>
-      </c>
-      <c r="J8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="P8" s="3" t="n">
-        <v>156154.688999999</v>
-      </c>
-      <c r="Q8" s="3" t="n">
-        <v>87027.7005000003</v>
-      </c>
-      <c r="R8" s="3" t="n">
-        <v>1.89626322957643</v>
-      </c>
-      <c r="S8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="V8" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="W8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="X8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z8" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>7132</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="2" t="n">
-        <v>92660.11</v>
-      </c>
-      <c r="J9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="P9" s="3" t="n">
-        <v>209263.928099994</v>
-      </c>
-      <c r="Q9" s="3" t="n">
-        <v>116603.814600002</v>
-      </c>
-      <c r="R9" s="3" t="n">
-        <v>1.88845742716933</v>
-      </c>
-      <c r="S9" s="3" t="n">
-        <v>1828</v>
-      </c>
-      <c r="T9" s="3" t="n">
-        <v>23533.1249999935</v>
-      </c>
-      <c r="U9" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="V9" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="W9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="X9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z9" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:U10"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="21.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="27.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="13.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="14.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="24.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="21.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="19.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="20.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="30.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="27.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="19.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="20.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="30.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="27.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="17.29"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>36</v>
@@ -3426,7 +2665,7 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>36</v>
@@ -3434,7 +2673,7 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>36</v>
@@ -3443,299 +2682,139 @@
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9"/>
       <c r="B5" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="10" t="s">
         <v>37</v>
       </c>
+      <c r="C5" s="11"/>
       <c r="D5" s="11"/>
       <c r="E5" s="11"/>
       <c r="F5" s="11"/>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
       <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="11"/>
-      <c r="S5" s="11"/>
-      <c r="T5" s="11"/>
-      <c r="U5" s="12"/>
+      <c r="J5" s="12"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13"/>
+      <c r="A6" s="13" t="s">
+        <v>0</v>
+      </c>
       <c r="B6" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
+        <v>38</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>41</v>
+      </c>
       <c r="F6" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
-      <c r="M6" s="15"/>
-      <c r="N6" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="O6" s="15"/>
-      <c r="P6" s="15"/>
-      <c r="Q6" s="15"/>
-      <c r="R6" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="S6" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="T6" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="U6" s="17" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="I6" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="J6" s="16" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="D7" s="20" t="s">
-        <v>44</v>
-      </c>
-      <c r="E7" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="F7" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" s="20" t="s">
-        <v>44</v>
-      </c>
-      <c r="I7" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="J7" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="K7" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="L7" s="20" t="s">
-        <v>44</v>
-      </c>
-      <c r="M7" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="N7" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="O7" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="P7" s="20" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q7" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="R7" s="21"/>
-      <c r="S7" s="21"/>
-      <c r="T7" s="21"/>
-      <c r="U7" s="22"/>
+      <c r="A7" s="17" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B7" s="18" t="n">
+        <v>72460</v>
+      </c>
+      <c r="C7" s="19"/>
+      <c r="D7" s="20" t="n">
+        <v>6.07857142857143</v>
+      </c>
+      <c r="E7" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="21" t="n">
+        <v>121.448899447743</v>
+      </c>
+      <c r="H7" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B8" s="24" t="n">
-        <v>36230</v>
-      </c>
-      <c r="C8" s="25"/>
+        <v>90628</v>
+      </c>
+      <c r="C8" s="25" t="n">
+        <v>-0.0205095658740228</v>
+      </c>
       <c r="D8" s="26" t="n">
-        <v>42.55</v>
-      </c>
-      <c r="E8" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="28" t="n">
-        <v>25316</v>
-      </c>
-      <c r="G8" s="29"/>
-      <c r="H8" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="24" t="n">
-        <v>5610</v>
-      </c>
-      <c r="K8" s="25"/>
-      <c r="L8" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="28" t="n">
-        <v>5304</v>
-      </c>
-      <c r="O8" s="29"/>
-      <c r="P8" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="31" t="n">
-        <v>72460</v>
-      </c>
-      <c r="S8" s="32"/>
-      <c r="T8" s="33" t="n">
-        <v>10.6375</v>
-      </c>
-      <c r="U8" s="34" t="n">
-        <v>0</v>
+        <v>6.04857142857143</v>
+      </c>
+      <c r="E8" s="26" t="n">
+        <v>-0.305714285714286</v>
+      </c>
+      <c r="F8" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="27" t="n">
+        <v>92.1688397827653</v>
+      </c>
+      <c r="H8" s="26" t="n">
+        <v>-2.14</v>
+      </c>
+      <c r="I8" s="26" t="n">
+        <v>25.07</v>
+      </c>
+      <c r="J8" s="28" t="n">
+        <v>-78055.1521999448</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="35" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B9" s="36" t="n">
-        <v>45314</v>
-      </c>
-      <c r="C9" s="37" t="n">
-        <v>-0.0214058678606908</v>
-      </c>
-      <c r="D9" s="38" t="n">
-        <v>42.34</v>
-      </c>
-      <c r="E9" s="39" t="n">
+      <c r="A9" s="29" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="30" t="n">
+        <v>163088</v>
+      </c>
+      <c r="C9" s="31"/>
+      <c r="D9" s="32" t="n">
+        <v>6.06357142857143</v>
+      </c>
+      <c r="E9" s="32" t="n">
+        <v>-0.152857142857143</v>
+      </c>
+      <c r="F9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="33" t="n">
+        <v>106.808869615254</v>
+      </c>
+      <c r="H9" s="32" t="n">
         <v>-2.14</v>
       </c>
-      <c r="F9" s="28" t="n">
-        <v>32493</v>
-      </c>
-      <c r="G9" s="40" t="n">
-        <v>0.270538254915235</v>
-      </c>
-      <c r="H9" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="36" t="n">
-        <v>5689</v>
-      </c>
-      <c r="K9" s="37" t="n">
-        <v>-0.0464697349070941</v>
-      </c>
-      <c r="L9" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="28" t="n">
-        <v>7132</v>
-      </c>
-      <c r="O9" s="40" t="n">
-        <v>0.340433165106711</v>
-      </c>
-      <c r="P9" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" s="41" t="n">
-        <v>90628</v>
-      </c>
-      <c r="S9" s="42" t="n">
-        <v>-0.0205095658740228</v>
-      </c>
-      <c r="T9" s="43" t="n">
-        <v>10.585</v>
-      </c>
-      <c r="U9" s="44" t="n">
-        <v>-0.535</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="45" t="s">
-        <v>46</v>
-      </c>
-      <c r="B10" s="46" t="n">
-        <v>81544</v>
-      </c>
-      <c r="C10" s="47"/>
-      <c r="D10" s="48" t="n">
-        <v>42.445</v>
-      </c>
-      <c r="E10" s="49" t="n">
-        <v>-1.07</v>
-      </c>
-      <c r="F10" s="46" t="n">
-        <v>57809</v>
-      </c>
-      <c r="G10" s="47"/>
-      <c r="H10" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="46" t="n">
-        <v>11299</v>
-      </c>
-      <c r="K10" s="47"/>
-      <c r="L10" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="46" t="n">
-        <v>12436</v>
-      </c>
-      <c r="O10" s="47"/>
-      <c r="P10" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" s="50" t="n">
-        <v>163088</v>
-      </c>
-      <c r="S10" s="51"/>
-      <c r="T10" s="52" t="n">
-        <v>10.61125</v>
-      </c>
-      <c r="U10" s="53" t="n">
-        <v>-0.2675</v>
+      <c r="I9" s="32" t="n">
+        <v>25.07</v>
+      </c>
+      <c r="J9" s="34" t="n">
+        <v>-78055.1521999448</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Data Vizualitation for EDA 01 part 1
</commit_message>
<xml_diff>
--- a/Project-5-AdventureWorks-Sales-Performance-Analysis/excel/01_eda/01_decline_profit.xlsx
+++ b/Project-5-AdventureWorks-Sales-Performance-Analysis/excel/01_eda/01_decline_profit.xlsx
@@ -5,23 +5,24 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard_Index" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Viz_Dashboard" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="All_Data" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Pivot Table_All_Data_1" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="01_Top3_Decliners" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="02_Pacific_Crisis" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="03_YoY_Negative" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="04_Bikes_Drivers" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="05_High_Returns" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="06_Top2_2022_Fix" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="Data_For_Viz" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="All_Data" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Pivot Table_All_Data_1" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="01_Top3_Decliners" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="02_Pacific_Crisis" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="03_YoY_Negative" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="04_Bikes_Drivers" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="05_High_Returns" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="06_Top2_2022_Fix" sheetId="11" state="visible" r:id="rId13"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId14"/>
+    <pivotCache cacheId="1" r:id="rId15"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="103">
   <si>
     <t xml:space="preserve">AdventureWorks Profit Decline EDA - Dashboard Index</t>
   </si>
@@ -139,6 +140,60 @@
     <t xml:space="preserve">Profit Decline 2022 Viz</t>
   </si>
   <si>
+    <t xml:space="preserve">Metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YoY_Delta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YoY_Pct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profit_Delta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Continent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">net_sales_2022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">returns_per_qty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volume (Qty)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accessories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Europe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profit (Net)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bikes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">North America</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Margin %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clothing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pacific</t>
+  </si>
+  <si>
     <t xml:space="preserve">year</t>
   </si>
   <si>
@@ -211,9 +266,6 @@
     <t xml:space="preserve">net_sales_value</t>
   </si>
   <si>
-    <t xml:space="preserve">returns_per_qty</t>
-  </si>
-  <si>
     <t xml:space="preserve">source</t>
   </si>
   <si>
@@ -223,28 +275,10 @@
     <t xml:space="preserve">Overall</t>
   </si>
   <si>
-    <t xml:space="preserve">Accessories</t>
-  </si>
-  <si>
     <t xml:space="preserve">Categories</t>
   </si>
   <si>
-    <t xml:space="preserve">Bikes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clothing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Europe</t>
-  </si>
-  <si>
     <t xml:space="preserve">Territory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">North America</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pacific</t>
   </si>
   <si>
     <t xml:space="preserve">- all -</t>
@@ -314,12 +348,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0"/>
-    <numFmt numFmtId="166" formatCode="0.00"/>
+    <numFmt numFmtId="166" formatCode="0.00%"/>
+    <numFmt numFmtId="167" formatCode="0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -375,8 +410,25 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -387,6 +439,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF5983B0"/>
         <bgColor rgb="FF808080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF158466"/>
+        <bgColor rgb="FF008080"/>
       </patternFill>
     </fill>
   </fills>
@@ -701,7 +759,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="109">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -750,15 +808,43 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -766,7 +852,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -822,7 +908,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="16" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="16" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -842,7 +928,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="13" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="13" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -862,7 +948,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="21" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="21" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -930,7 +1016,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="16" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="16" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -954,7 +1040,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -978,7 +1064,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="13" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="13" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1002,7 +1088,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="21" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="21" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1034,15 +1120,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="32" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="33" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="28" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="32" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="33" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="28" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1136,12 +1222,12 @@
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF18A303"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF158466"/>
+      <rgbColor rgb="FFB3B3B3"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
@@ -1149,7 +1235,7 @@
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FF0369A3"/>
       <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -1175,17 +1261,950 @@
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF5983B0"/>
       <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF004D77"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FFA33E03"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1300" b="1" u="none" strike="noStrike">
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>Decline Drivers: Bikes -169K</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Data_For_Viz!$G$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Profit_Delta</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="004d77"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="004d77"/>
+              </a:solidFill>
+              <a:ln w="0">
+                <a:noFill/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="ff0000"/>
+              </a:solidFill>
+              <a:ln w="0">
+                <a:noFill/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:numFmt formatCode="0" sourceLinked="0"/>
+              <c:txPr>
+                <a:bodyPr wrap="none"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:uFillTx/>
+                      <a:latin typeface="Arial"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:separator> </c:separator>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:numFmt formatCode="0" sourceLinked="0"/>
+              <c:txPr>
+                <a:bodyPr wrap="none"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:uFillTx/>
+                      <a:latin typeface="Arial"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:separator> </c:separator>
+            </c:dLbl>
+            <c:numFmt formatCode="0" sourceLinked="0"/>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:uFillTx/>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="0">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                </a:ln>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Data_For_Viz!$F$2:$F$4</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Accessories</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Bikes</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Clothing</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Data_For_Viz!$G$2:$G$4</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>67888</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-169476</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>23533</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="100"/>
+        <c:overlap val="0"/>
+        <c:axId val="41136131"/>
+        <c:axId val="62277710"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="41136131"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="0">
+            <a:solidFill>
+              <a:srgbClr val="b3b3b3"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="62277710"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="62277710"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="b3b3b3"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="0">
+            <a:solidFill>
+              <a:srgbClr val="b3b3b3"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="41136131"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:solidFill>
+            <a:srgbClr val="b3b3b3"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+              <a:uFillTx/>
+              <a:latin typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="0">
+      <a:noFill/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1400" b="1" u="none" strike="noStrike">
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>Volume ↑25% vs Profit ↓2%</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Data_For_Viz!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2021</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="18a303"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="General" sourceLinked="1"/>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:uFillTx/>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="0">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                </a:ln>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Data_For_Viz!$A$2:$A$3</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Volume (Qty)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Profit (Net)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Data_For_Viz!$B$2:$B$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>36230</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3690735</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Data_For_Viz!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2022</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0369a3"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="General" sourceLinked="1"/>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:uFillTx/>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="0">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                </a:ln>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Data_For_Viz!$A$2:$A$3</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Volume (Qty)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Profit (Net)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Data_For_Viz!$C$2:$C$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>45314</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3611731</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="100"/>
+        <c:overlap val="0"/>
+        <c:axId val="8905746"/>
+        <c:axId val="65452323"/>
+      </c:barChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Data_For_Viz!$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>YoY_Pct</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="a33e03"/>
+            </a:solidFill>
+            <a:ln w="28800">
+              <a:solidFill>
+                <a:srgbClr val="a33e03"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:numFmt formatCode="0.00%" sourceLinked="1"/>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:uFillTx/>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="t"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="28800">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                </a:ln>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Data_For_Viz!$A$2:$A$3</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Volume (Qty)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Profit (Net)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Data_For_Viz!$E$2:$E$3</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0.2507</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.0214</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:hiLowLines>
+          <c:spPr>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:hiLowLines>
+        <c:marker val="0"/>
+        <c:axId val="9521995"/>
+        <c:axId val="93402037"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="8905746"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="0">
+            <a:solidFill>
+              <a:srgbClr val="b3b3b3"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="65452323"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="65452323"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="b3b3b3"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="0">
+            <a:solidFill>
+              <a:srgbClr val="b3b3b3"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="8905746"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:catAx>
+        <c:axId val="9521995"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="t"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="0">
+            <a:solidFill>
+              <a:srgbClr val="b3b3b3"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="93402037"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="93402037"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="r"/>
+        <c:numFmt formatCode="0.00%" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="0">
+            <a:solidFill>
+              <a:srgbClr val="b3b3b3"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="9521995"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:solidFill>
+            <a:srgbClr val="b3b3b3"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+              <a:uFillTx/>
+              <a:latin typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="0">
+      <a:noFill/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>198360</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>37080</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>39600</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>59760</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name=""/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="5887800" y="317160"/>
+        <a:ext cx="5531040" cy="3111120"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>792720</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>146520</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name=""/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="325800"/>
+        <a:ext cx="5669640" cy="3189240"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1904,13 +2923,13 @@
   </pageFields>
   <dataFields count="9">
     <dataField name="Sum - total_qty" fld="1" subtotal="sum" numFmtId="165"/>
-    <dataField name="Sum - net_profit" fld="8" subtotal="sum" numFmtId="166"/>
-    <dataField name="Average - gross_margin_pct" fld="13" subtotal="average" numFmtId="166"/>
-    <dataField name="Average - profit_yoy_pct" fld="12" subtotal="average" numFmtId="166"/>
+    <dataField name="Sum - net_profit" fld="8" subtotal="sum" numFmtId="167"/>
+    <dataField name="Average - gross_margin_pct" fld="13" subtotal="average" numFmtId="167"/>
+    <dataField name="Average - profit_yoy_pct" fld="12" subtotal="average" numFmtId="167"/>
     <dataField name="Min - decline_rank" fld="20" subtotal="min" numFmtId="164"/>
     <dataField name="Average - returns_per_qty" fld="24" subtotal="average" numFmtId="164"/>
-    <dataField name="Average - profit_yoy_pct" fld="12" subtotal="sum" numFmtId="166"/>
-    <dataField name="Sum - qty_yoy_pct" fld="11" subtotal="sum" numFmtId="166"/>
+    <dataField name="Average - profit_yoy_pct" fld="12" subtotal="sum" numFmtId="167"/>
+    <dataField name="Sum - qty_yoy_pct" fld="11" subtotal="sum" numFmtId="167"/>
     <dataField name="Sum - profit_delta" fld="19" subtotal="sum" numFmtId="164"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
@@ -2209,6 +3228,134 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A2:D11"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="22.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="28.56"/>
+  </cols>
+  <sheetData>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="50" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="50" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="50" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="93"/>
+      <c r="B5" s="94"/>
+      <c r="C5" s="94"/>
+      <c r="D5" s="95"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="96"/>
+      <c r="B6" s="53" t="s">
+        <v>74</v>
+      </c>
+      <c r="C6" s="97"/>
+      <c r="D6" s="52"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="98"/>
+      <c r="B7" s="99" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="100" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="101" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="57" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="59" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" s="59" t="s">
+        <v>89</v>
+      </c>
+      <c r="D8" s="102"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="103" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B9" s="65" t="n">
+        <v>284.275128347168</v>
+      </c>
+      <c r="C9" s="71" t="n">
+        <v>375.741416680663</v>
+      </c>
+      <c r="D9" s="104" t="n">
+        <v>330.008272513916</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="105" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B10" s="77" t="n">
+        <v>215.69839258202</v>
+      </c>
+      <c r="C10" s="71" t="n">
+        <v>253.814111575181</v>
+      </c>
+      <c r="D10" s="104" t="n">
+        <v>234.7562520786</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="106" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" s="107" t="n">
+        <v>249.986760464594</v>
+      </c>
+      <c r="C11" s="107" t="n">
+        <v>314.777764127922</v>
+      </c>
+      <c r="D11" s="108" t="n">
+        <v>282.382262296258</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A2:F10"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2222,111 +3369,111 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="43" t="s">
-        <v>64</v>
+        <v>77</v>
+      </c>
+      <c r="B2" s="50" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B3" s="43" t="s">
-        <v>83</v>
+        <v>93</v>
+      </c>
+      <c r="B3" s="50" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" s="43" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="50" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="51"/>
+      <c r="B6" s="52"/>
+      <c r="C6" s="53" t="s">
+        <v>83</v>
+      </c>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="55"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="56" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="57" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="58" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" s="59" t="s">
+        <v>85</v>
+      </c>
+      <c r="E7" s="59" t="s">
+        <v>88</v>
+      </c>
+      <c r="F7" s="60" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="44"/>
-      <c r="B6" s="45"/>
-      <c r="C6" s="46" t="s">
-        <v>72</v>
-      </c>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="48"/>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="49" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="50" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" s="51" t="s">
-        <v>73</v>
-      </c>
-      <c r="D7" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="E7" s="52" t="s">
-        <v>77</v>
-      </c>
-      <c r="F7" s="53" t="s">
-        <v>80</v>
-      </c>
-    </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="54" t="n">
+      <c r="A8" s="61" t="n">
         <v>2022</v>
       </c>
-      <c r="B8" s="55" t="s">
-        <v>65</v>
-      </c>
-      <c r="C8" s="56" t="n">
+      <c r="B8" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="63" t="n">
         <v>5689</v>
       </c>
-      <c r="D8" s="57" t="n">
+      <c r="D8" s="64" t="n">
         <v>3477544.92</v>
       </c>
-      <c r="E8" s="58" t="n">
+      <c r="E8" s="65" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="59" t="n">
+      <c r="F8" s="66" t="n">
         <v>-169476.092199898</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="66"/>
-      <c r="B9" s="67" t="s">
-        <v>66</v>
-      </c>
-      <c r="C9" s="68" t="n">
+      <c r="A9" s="73"/>
+      <c r="B9" s="74" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="75" t="n">
         <v>7132</v>
       </c>
-      <c r="D9" s="69" t="n">
+      <c r="D9" s="76" t="n">
         <v>92660.11</v>
       </c>
-      <c r="E9" s="70" t="n">
+      <c r="E9" s="77" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="71" t="n">
+      <c r="F9" s="78" t="n">
         <v>23533.1249999935</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="72" t="s">
-        <v>81</v>
-      </c>
-      <c r="B10" s="73"/>
-      <c r="C10" s="74" t="n">
+      <c r="A10" s="79" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="80"/>
+      <c r="C10" s="81" t="n">
         <v>12821</v>
       </c>
-      <c r="D10" s="75" t="n">
+      <c r="D10" s="82" t="n">
         <v>3570205.03</v>
       </c>
-      <c r="E10" s="76" t="n">
+      <c r="E10" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="77" t="n">
+      <c r="F10" s="84" t="n">
         <v>-145942.967199905</v>
       </c>
     </row>
@@ -2368,6 +3515,7 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2376,16 +3524,185 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="8.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="5.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="13.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="14.09"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="13" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C1" s="13" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="J1" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="K1" s="13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="14" t="n">
+        <v>36230</v>
+      </c>
+      <c r="C2" s="14" t="n">
+        <v>45314</v>
+      </c>
+      <c r="D2" s="15" t="n">
+        <v>9084</v>
+      </c>
+      <c r="E2" s="16" t="n">
+        <v>0.2507</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" s="15" t="n">
+        <v>67888</v>
+      </c>
+      <c r="H2" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="I2" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="J2" s="18" t="n">
+        <v>3218911</v>
+      </c>
+      <c r="K2" s="19" t="n">
+        <v>215.7</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="14" t="n">
+        <v>3690735</v>
+      </c>
+      <c r="C3" s="14" t="n">
+        <v>3611731</v>
+      </c>
+      <c r="D3" s="15" t="n">
+        <v>-7904</v>
+      </c>
+      <c r="E3" s="16" t="n">
+        <v>-0.0214</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3" s="15" t="n">
+        <v>-169476</v>
+      </c>
+      <c r="H3" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="J3" s="18" t="n">
+        <v>3293497</v>
+      </c>
+      <c r="K3" s="19" t="n">
+        <v>175.67</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" s="16" t="n">
+        <v>0.4255</v>
+      </c>
+      <c r="C4" s="16" t="n">
+        <v>0.4234</v>
+      </c>
+      <c r="D4" s="16" t="n">
+        <v>-0.0021</v>
+      </c>
+      <c r="E4" s="16" t="n">
+        <v>-0.0049</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" s="15" t="n">
+        <v>23533</v>
+      </c>
+      <c r="H4" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="J4" s="18" t="n">
+        <v>34931</v>
+      </c>
+      <c r="K4" s="19" t="n">
+        <v>253.81</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:Z50"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="13" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="14" width="13.4"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="4" style="14" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="14" width="16.74"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="12" min="7" style="14" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="14" width="12.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="14" width="15.9"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="20" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="21" width="13.4"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="4" style="21" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="21" width="16.74"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="12" min="7" style="21" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="21" width="12.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="21" width="15.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="13.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="13.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="13.12"/>
@@ -2394,290 +3711,290 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="B1" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="E1" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="F1" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="G1" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="H1" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="I1" s="16" t="s">
+      <c r="A1" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="G1" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="H1" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="I1" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="J1" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="L1" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="M1" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="N1" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="O1" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="P1" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q1" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="R1" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="S1" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="T1" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="U1" s="24" t="s">
+        <v>73</v>
+      </c>
+      <c r="V1" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="W1" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="X1" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y1" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="J1" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="K1" s="16" t="s">
+      <c r="Z1" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="22" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B2" s="22" t="n">
+        <v>36230</v>
+      </c>
+      <c r="C2" s="21" t="n">
+        <v>9324203.79</v>
+      </c>
+      <c r="D2" s="21" t="n">
+        <v>5357119.66</v>
+      </c>
+      <c r="E2" s="21" t="n">
+        <v>3967084.13</v>
+      </c>
+      <c r="F2" s="21" t="n">
+        <v>770</v>
+      </c>
+      <c r="G2" s="21" t="n">
+        <v>276348.93</v>
+      </c>
+      <c r="H2" s="21" t="n">
+        <v>35460</v>
+      </c>
+      <c r="I2" s="21" t="n">
+        <v>3690735.2</v>
+      </c>
+      <c r="J2" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="21" t="n">
+        <v>42.55</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="P2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="W2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="22" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B3" s="22" t="n">
+        <v>45314</v>
+      </c>
+      <c r="C3" s="21" t="n">
+        <v>9185449.45</v>
+      </c>
+      <c r="D3" s="21" t="n">
+        <v>5296420.47</v>
+      </c>
+      <c r="E3" s="21" t="n">
+        <v>3889028.97</v>
+      </c>
+      <c r="F3" s="21" t="n">
+        <v>972</v>
+      </c>
+      <c r="G3" s="21" t="n">
+        <v>277297.17</v>
+      </c>
+      <c r="H3" s="21" t="n">
+        <v>44342</v>
+      </c>
+      <c r="I3" s="21" t="n">
+        <v>3611731.81</v>
+      </c>
+      <c r="J3" s="21" t="n">
+        <v>36230</v>
+      </c>
+      <c r="K3" s="21" t="n">
+        <v>3690735.2</v>
+      </c>
+      <c r="L3" s="21" t="n">
+        <v>25.07</v>
+      </c>
+      <c r="M3" s="21" t="n">
+        <v>-2.14</v>
+      </c>
+      <c r="N3" s="21" t="n">
+        <v>42.34</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="P3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="W3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="22" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B4" s="22" t="n">
+        <v>25316</v>
+      </c>
+      <c r="C4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="21" t="n">
+        <v>250936.12</v>
+      </c>
+      <c r="J4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="L1" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="M1" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="N1" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="O1" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="P1" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q1" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="R1" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="S1" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="T1" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="U1" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="V1" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="W1" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="X1" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y1" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="Z1" s="17" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="15" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B2" s="15" t="n">
-        <v>36230</v>
-      </c>
-      <c r="C2" s="14" t="n">
-        <v>9324203.79</v>
-      </c>
-      <c r="D2" s="14" t="n">
-        <v>5357119.66</v>
-      </c>
-      <c r="E2" s="14" t="n">
-        <v>3967084.13</v>
-      </c>
-      <c r="F2" s="14" t="n">
-        <v>770</v>
-      </c>
-      <c r="G2" s="14" t="n">
-        <v>276348.93</v>
-      </c>
-      <c r="H2" s="14" t="n">
-        <v>35460</v>
-      </c>
-      <c r="I2" s="14" t="n">
-        <v>3690735.2</v>
-      </c>
-      <c r="J2" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="14" t="n">
-        <v>42.55</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="P2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="W2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="X2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B3" s="15" t="n">
-        <v>45314</v>
-      </c>
-      <c r="C3" s="14" t="n">
-        <v>9185449.45</v>
-      </c>
-      <c r="D3" s="14" t="n">
-        <v>5296420.47</v>
-      </c>
-      <c r="E3" s="14" t="n">
-        <v>3889028.97</v>
-      </c>
-      <c r="F3" s="14" t="n">
-        <v>972</v>
-      </c>
-      <c r="G3" s="14" t="n">
-        <v>277297.17</v>
-      </c>
-      <c r="H3" s="14" t="n">
-        <v>44342</v>
-      </c>
-      <c r="I3" s="14" t="n">
-        <v>3611731.81</v>
-      </c>
-      <c r="J3" s="14" t="n">
-        <v>36230</v>
-      </c>
-      <c r="K3" s="14" t="n">
-        <v>3690735.2</v>
-      </c>
-      <c r="L3" s="14" t="n">
-        <v>25.07</v>
-      </c>
-      <c r="M3" s="14" t="n">
-        <v>-2.14</v>
-      </c>
-      <c r="N3" s="14" t="n">
-        <v>42.34</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="P3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="U3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="V3" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="W3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="X3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z3" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B4" s="15" t="n">
-        <v>25316</v>
-      </c>
-      <c r="C4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="14" t="n">
-        <v>250936.12</v>
-      </c>
-      <c r="J4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="P4" s="1" t="n">
         <v>399342.117799956</v>
@@ -2698,7 +4015,7 @@
         <v>6</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="W4" s="1" t="n">
         <v>0</v>
@@ -2710,54 +4027,54 @@
         <v>0</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="n">
+      <c r="A5" s="22" t="n">
         <v>2022</v>
       </c>
-      <c r="B5" s="15" t="n">
+      <c r="B5" s="22" t="n">
         <v>32493</v>
       </c>
-      <c r="C5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="14" t="n">
+      <c r="C5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="21" t="n">
         <v>318823.94</v>
       </c>
-      <c r="J5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="14" t="n">
+      <c r="J5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="21" t="n">
         <v>0</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="P5" s="1" t="n">
         <v>507330.989199908</v>
@@ -2778,7 +4095,7 @@
         <v>3</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="W5" s="1" t="n">
         <v>0</v>
@@ -2790,54 +4107,54 @@
         <v>0</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="n">
+      <c r="A6" s="22" t="n">
         <v>2021</v>
       </c>
-      <c r="B6" s="15" t="n">
+      <c r="B6" s="22" t="n">
         <v>5610</v>
       </c>
-      <c r="C6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="14" t="n">
+      <c r="C6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="21" t="n">
         <v>3647021.02</v>
       </c>
-      <c r="J6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="14" t="n">
+      <c r="J6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="21" t="n">
         <v>0</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="P6" s="1" t="n">
         <v>8768706.98490015</v>
@@ -2858,7 +4175,7 @@
         <v>4</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="W6" s="1" t="n">
         <v>0</v>
@@ -2870,54 +4187,54 @@
         <v>0</v>
       </c>
       <c r="Z6" s="1" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="n">
+      <c r="A7" s="22" t="n">
         <v>2022</v>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="22" t="n">
         <v>5689</v>
       </c>
-      <c r="C7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="14" t="n">
+      <c r="C7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="21" t="n">
         <v>3477544.92</v>
       </c>
-      <c r="J7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="14" t="n">
+      <c r="J7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="21" t="n">
         <v>0</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="P7" s="1" t="n">
         <v>8468854.53000019</v>
@@ -2938,7 +4255,7 @@
         <v>1</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="W7" s="1" t="n">
         <v>0</v>
@@ -2950,54 +4267,54 @@
         <v>0</v>
       </c>
       <c r="Z7" s="1" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="n">
+      <c r="A8" s="22" t="n">
         <v>2021</v>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="22" t="n">
         <v>5304</v>
       </c>
-      <c r="C8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="14" t="n">
+      <c r="C8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="21" t="n">
         <v>69126.99</v>
       </c>
-      <c r="J8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="14" t="n">
+      <c r="J8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="21" t="n">
         <v>0</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="P8" s="1" t="n">
         <v>156154.688999999</v>
@@ -3018,7 +4335,7 @@
         <v>5</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="W8" s="1" t="n">
         <v>0</v>
@@ -3030,54 +4347,54 @@
         <v>0</v>
       </c>
       <c r="Z8" s="1" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="n">
+      <c r="A9" s="22" t="n">
         <v>2022</v>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="22" t="n">
         <v>7132</v>
       </c>
-      <c r="C9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="14" t="n">
+      <c r="C9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="21" t="n">
         <v>92660.11</v>
       </c>
-      <c r="J9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="14" t="n">
+      <c r="J9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="21" t="n">
         <v>0</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="P9" s="1" t="n">
         <v>209263.928099994</v>
@@ -3098,7 +4415,7 @@
         <v>2</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="W9" s="1" t="n">
         <v>0</v>
@@ -3110,54 +4427,54 @@
         <v>0</v>
       </c>
       <c r="Z9" s="1" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="n">
+      <c r="A10" s="22" t="n">
         <v>2021</v>
       </c>
-      <c r="B10" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="14" t="n">
+      <c r="B10" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="21" t="n">
         <v>0</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="P10" s="1" t="n">
         <v>0</v>
@@ -3178,7 +4495,7 @@
         <v>0</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="W10" s="1" t="n">
         <v>864233</v>
@@ -3190,54 +4507,54 @@
         <v>284.275128347168</v>
       </c>
       <c r="Z10" s="1" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="n">
+      <c r="A11" s="22" t="n">
         <v>2021</v>
       </c>
-      <c r="B11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="14" t="n">
+      <c r="B11" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="21" t="n">
         <v>0</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="P11" s="1" t="n">
         <v>0</v>
@@ -3258,7 +4575,7 @@
         <v>0</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="W11" s="1" t="n">
         <v>2218218</v>
@@ -3270,54 +4587,54 @@
         <v>190.12575110637</v>
       </c>
       <c r="Z11" s="1" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="n">
+      <c r="A12" s="22" t="n">
         <v>2021</v>
       </c>
-      <c r="B12" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="14" t="n">
+      <c r="B12" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="21" t="n">
         <v>0</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="P12" s="1" t="n">
         <v>0</v>
@@ -3338,7 +4655,7 @@
         <v>0</v>
       </c>
       <c r="V12" s="1" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="W12" s="1" t="n">
         <v>1249024</v>
@@ -3350,54 +4667,54 @@
         <v>375.741416680663</v>
       </c>
       <c r="Z12" s="1" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="n">
+      <c r="A13" s="22" t="n">
         <v>2022</v>
       </c>
-      <c r="B13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="14" t="n">
+      <c r="B13" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="21" t="n">
         <v>0</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="P13" s="1" t="n">
         <v>0</v>
@@ -3418,7 +4735,7 @@
         <v>0</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="W13" s="1" t="n">
         <v>1353420</v>
@@ -3430,54 +4747,54 @@
         <v>215.69839258202</v>
       </c>
       <c r="Z13" s="1" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="n">
+      <c r="A14" s="22" t="n">
         <v>2022</v>
       </c>
-      <c r="B14" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="14" t="n">
+      <c r="B14" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="21" t="n">
         <v>0</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="P14" s="1" t="n">
         <v>0</v>
@@ -3498,7 +4815,7 @@
         <v>0</v>
       </c>
       <c r="V14" s="1" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="W14" s="1" t="n">
         <v>3496046</v>
@@ -3510,54 +4827,54 @@
         <v>175.669374322156</v>
       </c>
       <c r="Z14" s="1" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="n">
+      <c r="A15" s="22" t="n">
         <v>2022</v>
       </c>
-      <c r="B15" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="14" t="n">
+      <c r="B15" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="21" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="P15" s="1" t="n">
         <v>0</v>
@@ -3578,7 +4895,7 @@
         <v>0</v>
       </c>
       <c r="V15" s="1" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="W15" s="1" t="n">
         <v>1944835</v>
@@ -3590,14 +4907,14 @@
         <v>253.814111575181</v>
       </c>
       <c r="Z15" s="1" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="15"/>
+      <c r="B20" s="22"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="15"/>
+      <c r="B50" s="22"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3610,7 +4927,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3658,11 +4975,11 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="19" t="s">
-        <v>71</v>
+      <c r="A2" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>82</v>
       </c>
       <c r="C2" s="0"/>
       <c r="D2" s="0"/>
@@ -3674,11 +4991,11 @@
       <c r="J2" s="0"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>71</v>
+      <c r="A3" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>82</v>
       </c>
       <c r="C3" s="0"/>
       <c r="D3" s="0"/>
@@ -3690,11 +5007,11 @@
       <c r="J3" s="0"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>71</v>
+      <c r="A4" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>82</v>
       </c>
       <c r="C4" s="0"/>
       <c r="D4" s="0"/>
@@ -3718,144 +5035,144 @@
       <c r="J5" s="0"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20"/>
-      <c r="B6" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="23"/>
+      <c r="A6" s="27"/>
+      <c r="B6" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="29"/>
+      <c r="I6" s="29"/>
+      <c r="J6" s="30"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="25" t="s">
-        <v>73</v>
-      </c>
-      <c r="C7" s="26" t="s">
-        <v>74</v>
-      </c>
-      <c r="D7" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="E7" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="F7" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="G7" s="26" t="s">
-        <v>78</v>
-      </c>
-      <c r="H7" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="I7" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="J7" s="27" t="s">
-        <v>80</v>
+      <c r="A7" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="33" t="s">
+        <v>85</v>
+      </c>
+      <c r="D7" s="33" t="s">
+        <v>86</v>
+      </c>
+      <c r="E7" s="33" t="s">
+        <v>87</v>
+      </c>
+      <c r="F7" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="G7" s="33" t="s">
+        <v>89</v>
+      </c>
+      <c r="H7" s="33" t="s">
+        <v>87</v>
+      </c>
+      <c r="I7" s="33" t="s">
+        <v>90</v>
+      </c>
+      <c r="J7" s="34" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28" t="n">
+      <c r="A8" s="35" t="n">
         <v>2021</v>
       </c>
-      <c r="B8" s="29" t="n">
+      <c r="B8" s="36" t="n">
         <v>72460</v>
       </c>
-      <c r="C8" s="30" t="n">
+      <c r="C8" s="37" t="n">
         <v>7657819.33</v>
       </c>
-      <c r="D8" s="30" t="n">
+      <c r="D8" s="37" t="n">
         <v>6.07857142857143</v>
       </c>
-      <c r="E8" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="31" t="n">
+      <c r="E8" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="38" t="n">
         <v>121.448899447743</v>
       </c>
-      <c r="H8" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="32" t="n">
+      <c r="H8" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="39" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="33" t="n">
+      <c r="A9" s="40" t="n">
         <v>2022</v>
       </c>
-      <c r="B9" s="34" t="n">
+      <c r="B9" s="41" t="n">
         <v>90628</v>
       </c>
-      <c r="C9" s="35" t="n">
+      <c r="C9" s="42" t="n">
         <v>7500760.78</v>
       </c>
-      <c r="D9" s="35" t="n">
+      <c r="D9" s="42" t="n">
         <v>6.04857142857143</v>
       </c>
-      <c r="E9" s="35" t="n">
+      <c r="E9" s="42" t="n">
         <v>-0.305714285714286</v>
       </c>
-      <c r="F9" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="36" t="n">
+      <c r="F9" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="43" t="n">
         <v>92.1688397827653</v>
       </c>
-      <c r="H9" s="35" t="n">
+      <c r="H9" s="42" t="n">
         <v>-2.14</v>
       </c>
-      <c r="I9" s="35" t="n">
+      <c r="I9" s="42" t="n">
         <v>25.07</v>
       </c>
-      <c r="J9" s="37" t="n">
+      <c r="J9" s="44" t="n">
         <v>-78055.1521999448</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="38" t="s">
-        <v>81</v>
-      </c>
-      <c r="B10" s="39" t="n">
+      <c r="A10" s="45" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="46" t="n">
         <v>163088</v>
       </c>
-      <c r="C10" s="40" t="n">
+      <c r="C10" s="47" t="n">
         <v>15158580.11</v>
       </c>
-      <c r="D10" s="40" t="n">
+      <c r="D10" s="47" t="n">
         <v>6.06357142857143</v>
       </c>
-      <c r="E10" s="40" t="n">
+      <c r="E10" s="47" t="n">
         <v>-0.152857142857143</v>
       </c>
-      <c r="F10" s="41" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="41" t="n">
+      <c r="F10" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="48" t="n">
         <v>106.808869615254</v>
       </c>
-      <c r="H10" s="40" t="n">
+      <c r="H10" s="47" t="n">
         <v>-2.14</v>
       </c>
-      <c r="I10" s="40" t="n">
+      <c r="I10" s="47" t="n">
         <v>25.07</v>
       </c>
-      <c r="J10" s="42" t="n">
+      <c r="J10" s="49" t="n">
         <v>-78055.1521999448</v>
       </c>
     </row>
@@ -3870,7 +5187,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3888,129 +5205,129 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="43" t="s">
-        <v>64</v>
+        <v>77</v>
+      </c>
+      <c r="B2" s="50" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B3" s="43" t="s">
-        <v>83</v>
+        <v>93</v>
+      </c>
+      <c r="B3" s="50" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" s="43" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="50" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="51"/>
+      <c r="B6" s="52"/>
+      <c r="C6" s="53" t="s">
+        <v>83</v>
+      </c>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="55"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="56" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="57" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="58" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="44"/>
-      <c r="B6" s="45"/>
-      <c r="C6" s="46" t="s">
-        <v>72</v>
-      </c>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="48"/>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="49" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="50" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" s="51" t="s">
-        <v>73</v>
-      </c>
-      <c r="D7" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="E7" s="52" t="s">
-        <v>77</v>
-      </c>
-      <c r="F7" s="53" t="s">
-        <v>80</v>
+      <c r="D7" s="59" t="s">
+        <v>85</v>
+      </c>
+      <c r="E7" s="59" t="s">
+        <v>88</v>
+      </c>
+      <c r="F7" s="60" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="54" t="n">
+      <c r="A8" s="61" t="n">
         <v>2022</v>
       </c>
-      <c r="B8" s="55" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8" s="56" t="n">
+      <c r="B8" s="62" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="63" t="n">
         <v>32493</v>
       </c>
-      <c r="D8" s="57" t="n">
+      <c r="D8" s="64" t="n">
         <v>318823.94</v>
       </c>
-      <c r="E8" s="58" t="n">
+      <c r="E8" s="65" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="59" t="n">
+      <c r="F8" s="66" t="n">
         <v>67887.8149999597</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="60"/>
-      <c r="B9" s="61" t="s">
-        <v>65</v>
-      </c>
-      <c r="C9" s="62" t="n">
+      <c r="A9" s="67"/>
+      <c r="B9" s="68" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" s="69" t="n">
         <v>5689</v>
       </c>
-      <c r="D9" s="63" t="n">
+      <c r="D9" s="70" t="n">
         <v>3477544.92</v>
       </c>
-      <c r="E9" s="64" t="n">
+      <c r="E9" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="65" t="n">
+      <c r="F9" s="72" t="n">
         <v>-169476.092199898</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="66"/>
-      <c r="B10" s="67" t="s">
-        <v>66</v>
-      </c>
-      <c r="C10" s="68" t="n">
+      <c r="A10" s="73"/>
+      <c r="B10" s="74" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="75" t="n">
         <v>7132</v>
       </c>
-      <c r="D10" s="69" t="n">
+      <c r="D10" s="76" t="n">
         <v>92660.11</v>
       </c>
-      <c r="E10" s="70" t="n">
+      <c r="E10" s="77" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="71" t="n">
+      <c r="F10" s="78" t="n">
         <v>23533.1249999935</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="72" t="s">
-        <v>81</v>
-      </c>
-      <c r="B11" s="73"/>
-      <c r="C11" s="74" t="n">
+      <c r="A11" s="79" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" s="80"/>
+      <c r="C11" s="81" t="n">
         <v>45314</v>
       </c>
-      <c r="D11" s="75" t="n">
+      <c r="D11" s="82" t="n">
         <v>3889028.97</v>
       </c>
-      <c r="E11" s="76" t="n">
+      <c r="E11" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="77" t="n">
+      <c r="F11" s="84" t="n">
         <v>-78055.1521999448</v>
       </c>
     </row>
@@ -4025,7 +5342,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -4040,74 +5357,74 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="43" t="s">
-        <v>68</v>
+        <v>77</v>
+      </c>
+      <c r="B2" s="50" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B3" s="43" t="s">
-        <v>70</v>
+        <v>93</v>
+      </c>
+      <c r="B3" s="50" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" s="43" t="s">
-        <v>83</v>
+        <v>73</v>
+      </c>
+      <c r="B4" s="50" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="78"/>
-      <c r="B6" s="47"/>
-      <c r="C6" s="48"/>
+      <c r="A6" s="85"/>
+      <c r="B6" s="54"/>
+      <c r="C6" s="55"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="49" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="52" t="s">
-        <v>78</v>
-      </c>
-      <c r="C7" s="53" t="s">
-        <v>85</v>
+      <c r="A7" s="56" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="59" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" s="60" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="54" t="n">
+      <c r="A8" s="61" t="n">
         <v>2021</v>
       </c>
-      <c r="B8" s="58" t="n">
+      <c r="B8" s="65" t="n">
         <v>375.741416680663</v>
       </c>
-      <c r="C8" s="59" t="n">
+      <c r="C8" s="66" t="n">
         <v>4270567.72329797</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="60" t="n">
+      <c r="A9" s="67" t="n">
         <v>2022</v>
       </c>
-      <c r="B9" s="70" t="n">
+      <c r="B9" s="77" t="n">
         <v>253.814111575181</v>
       </c>
-      <c r="C9" s="71" t="n">
+      <c r="C9" s="78" t="n">
         <v>34930.8751287839</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="79" t="s">
-        <v>81</v>
-      </c>
-      <c r="B10" s="76" t="n">
+      <c r="A10" s="86" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="83" t="n">
         <v>314.777764127922</v>
       </c>
-      <c r="C10" s="77" t="n">
+      <c r="C10" s="84" t="n">
         <v>4305498.59842676</v>
       </c>
     </row>
@@ -4122,7 +5439,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -4140,105 +5457,105 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="43" t="s">
-        <v>68</v>
+        <v>77</v>
+      </c>
+      <c r="B2" s="50" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B3" s="43" t="s">
-        <v>70</v>
+        <v>93</v>
+      </c>
+      <c r="B3" s="50" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" s="50" t="n">
+        <v>-2.14</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="85"/>
+      <c r="B6" s="53" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="54"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="87"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="56" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="58" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="59" t="s">
+        <v>85</v>
+      </c>
+      <c r="D7" s="59" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="43" t="n">
+      <c r="E7" s="59" t="s">
+        <v>87</v>
+      </c>
+      <c r="F7" s="59" t="s">
+        <v>87</v>
+      </c>
+      <c r="G7" s="88" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="61" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B8" s="89" t="n">
+        <v>45314</v>
+      </c>
+      <c r="C8" s="90" t="n">
+        <v>3611731.81</v>
+      </c>
+      <c r="D8" s="90" t="n">
+        <v>42.34</v>
+      </c>
+      <c r="E8" s="90" t="n">
         <v>-2.14</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="78"/>
-      <c r="B6" s="46" t="s">
-        <v>72</v>
-      </c>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="47"/>
-      <c r="G6" s="80"/>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="49" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="51" t="s">
-        <v>73</v>
-      </c>
-      <c r="C7" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="D7" s="52" t="s">
-        <v>75</v>
-      </c>
-      <c r="E7" s="52" t="s">
-        <v>76</v>
-      </c>
-      <c r="F7" s="52" t="s">
-        <v>76</v>
-      </c>
-      <c r="G7" s="81" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="54" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B8" s="82" t="n">
+      <c r="F8" s="90" t="n">
+        <v>-2.14</v>
+      </c>
+      <c r="G8" s="91" t="n">
+        <v>25.07</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="86" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" s="81" t="n">
         <v>45314</v>
       </c>
-      <c r="C8" s="83" t="n">
+      <c r="C9" s="82" t="n">
         <v>3611731.81</v>
       </c>
-      <c r="D8" s="83" t="n">
+      <c r="D9" s="82" t="n">
         <v>42.34</v>
       </c>
-      <c r="E8" s="83" t="n">
+      <c r="E9" s="82" t="n">
         <v>-2.14</v>
       </c>
-      <c r="F8" s="83" t="n">
+      <c r="F9" s="82" t="n">
         <v>-2.14</v>
       </c>
-      <c r="G8" s="84" t="n">
-        <v>25.07</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="79" t="s">
-        <v>81</v>
-      </c>
-      <c r="B9" s="74" t="n">
-        <v>45314</v>
-      </c>
-      <c r="C9" s="75" t="n">
-        <v>3611731.81</v>
-      </c>
-      <c r="D9" s="75" t="n">
-        <v>42.34</v>
-      </c>
-      <c r="E9" s="75" t="n">
-        <v>-2.14</v>
-      </c>
-      <c r="F9" s="75" t="n">
-        <v>-2.14</v>
-      </c>
-      <c r="G9" s="85" t="n">
+      <c r="G9" s="92" t="n">
         <v>25.07</v>
       </c>
     </row>
@@ -4253,7 +5570,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -4271,244 +5588,116 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="43" t="s">
-        <v>64</v>
+        <v>77</v>
+      </c>
+      <c r="B2" s="50" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B3" s="43" t="s">
-        <v>83</v>
+        <v>93</v>
+      </c>
+      <c r="B3" s="50" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B4" s="43" t="s">
-        <v>65</v>
+        <v>98</v>
+      </c>
+      <c r="B4" s="50" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="78"/>
-      <c r="B6" s="46" t="s">
-        <v>72</v>
-      </c>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="48"/>
+      <c r="A6" s="85"/>
+      <c r="B6" s="53" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="54"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="55"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="49" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="51" t="s">
-        <v>73</v>
-      </c>
-      <c r="C7" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="D7" s="52" t="s">
-        <v>77</v>
-      </c>
-      <c r="E7" s="52" t="s">
-        <v>80</v>
-      </c>
-      <c r="F7" s="53" t="s">
+      <c r="A7" s="56" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="58" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="59" t="s">
+        <v>85</v>
+      </c>
+      <c r="D7" s="59" t="s">
         <v>88</v>
       </c>
+      <c r="E7" s="59" t="s">
+        <v>91</v>
+      </c>
+      <c r="F7" s="60" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="54" t="n">
+      <c r="A8" s="61" t="n">
         <v>2021</v>
       </c>
-      <c r="B8" s="56" t="n">
+      <c r="B8" s="63" t="n">
         <v>5610</v>
       </c>
-      <c r="C8" s="57" t="n">
+      <c r="C8" s="64" t="n">
         <v>3647021.02</v>
       </c>
-      <c r="D8" s="58" t="n">
+      <c r="D8" s="65" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="58" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="59" t="n">
+      <c r="E8" s="65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="66" t="n">
         <v>1.70568672635527</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="60" t="n">
+      <c r="A9" s="67" t="n">
         <v>2022</v>
       </c>
-      <c r="B9" s="68" t="n">
+      <c r="B9" s="75" t="n">
         <v>5689</v>
       </c>
-      <c r="C9" s="69" t="n">
+      <c r="C9" s="76" t="n">
         <v>3477544.92</v>
       </c>
-      <c r="D9" s="70" t="n">
+      <c r="D9" s="77" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="70" t="n">
+      <c r="E9" s="77" t="n">
         <v>-169476.092199898</v>
       </c>
-      <c r="F9" s="71" t="n">
+      <c r="F9" s="78" t="n">
         <v>1.6921437844365</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="79" t="s">
-        <v>81</v>
-      </c>
-      <c r="B10" s="74" t="n">
+      <c r="A10" s="86" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="81" t="n">
         <v>11299</v>
       </c>
-      <c r="C10" s="75" t="n">
+      <c r="C10" s="82" t="n">
         <v>7124565.94</v>
       </c>
-      <c r="D10" s="76" t="n">
+      <c r="D10" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="76" t="n">
+      <c r="E10" s="83" t="n">
         <v>-169476.092199898</v>
       </c>
-      <c r="F10" s="77" t="n">
+      <c r="F10" s="84" t="n">
         <v>3.39783051079177</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A2:D11"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="22.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="28.56"/>
-  </cols>
-  <sheetData>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="43" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B3" s="43" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" s="43" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="86"/>
-      <c r="B5" s="87"/>
-      <c r="C5" s="87"/>
-      <c r="D5" s="88"/>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="89"/>
-      <c r="B6" s="46" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6" s="90"/>
-      <c r="D6" s="45"/>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="91"/>
-      <c r="B7" s="92" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" s="93" t="s">
-        <v>70</v>
-      </c>
-      <c r="D7" s="94" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="50" t="s">
-        <v>35</v>
-      </c>
-      <c r="B8" s="52" t="s">
-        <v>78</v>
-      </c>
-      <c r="C8" s="52" t="s">
-        <v>78</v>
-      </c>
-      <c r="D8" s="95"/>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="96" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B9" s="58" t="n">
-        <v>284.275128347168</v>
-      </c>
-      <c r="C9" s="64" t="n">
-        <v>375.741416680663</v>
-      </c>
-      <c r="D9" s="97" t="n">
-        <v>330.008272513916</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="98" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B10" s="70" t="n">
-        <v>215.69839258202</v>
-      </c>
-      <c r="C10" s="64" t="n">
-        <v>253.814111575181</v>
-      </c>
-      <c r="D10" s="97" t="n">
-        <v>234.7562520786</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="99" t="s">
-        <v>81</v>
-      </c>
-      <c r="B11" s="100" t="n">
-        <v>249.986760464594</v>
-      </c>
-      <c r="C11" s="100" t="n">
-        <v>314.777764127922</v>
-      </c>
-      <c r="D11" s="101" t="n">
-        <v>282.382262296258</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding a hyperlink in dashboard
</commit_message>
<xml_diff>
--- a/Project-5-AdventureWorks-Sales-Performance-Analysis/excel/01_eda/01_decline_profit.xlsx
+++ b/Project-5-AdventureWorks-Sales-Performance-Analysis/excel/01_eda/01_decline_profit.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard_Index" sheetId="1" state="visible" r:id="rId3"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="98">
   <si>
     <t xml:space="preserve">AdventureWorks Profit Decline EDA - Dashboard Index</t>
   </si>
@@ -56,9 +56,6 @@
     <t xml:space="preserve">Status</t>
   </si>
   <si>
-    <t xml:space="preserve">01_Top3_Decliners</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bikes rank1: Profit delta -Rp169K (margin ↓1.70→1.69)</t>
   </si>
   <si>
@@ -71,9 +68,6 @@
     <t xml:space="preserve">High</t>
   </si>
   <si>
-    <t xml:space="preserve">02_Pacific_Crisis</t>
-  </si>
-  <si>
     <t xml:space="preserve">net_sales 2022 Rp34K (vs Rp4.2jt 2021), returns 253/unit</t>
   </si>
   <si>
@@ -83,9 +77,6 @@
     <t xml:space="preserve">Quality control &amp; no-return policy Pacific</t>
   </si>
   <si>
-    <t xml:space="preserve">03_YoY_Negative</t>
-  </si>
-  <si>
     <t xml:space="preserve">Overall profit -2.14% despite volume +25%</t>
   </si>
   <si>
@@ -98,9 +89,6 @@
     <t xml:space="preserve">Medium</t>
   </si>
   <si>
-    <t xml:space="preserve">04_Bikes_Drivers</t>
-  </si>
-  <si>
     <t xml:space="preserve">Volume +79 but profit -169K, margin erosion</t>
   </si>
   <si>
@@ -110,9 +98,6 @@
     <t xml:space="preserve">Rise the price of Bikes by 2-3%</t>
   </si>
   <si>
-    <t xml:space="preserve">05_High_Returns</t>
-  </si>
-  <si>
     <t xml:space="preserve">Pacific is always &gt;250/unit (highest)</t>
   </si>
   <si>
@@ -120,9 +105,6 @@
   </si>
   <si>
     <t xml:space="preserve">Targeted promo/inspection</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06_Top2_2022_Fix</t>
   </si>
   <si>
     <t xml:space="preserve">Bikes down vs Clothing up +23K</t>
@@ -357,7 +339,7 @@
     <numFmt numFmtId="166" formatCode="0.00"/>
     <numFmt numFmtId="167" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="17">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -449,17 +431,14 @@
     <font>
       <b val="true"/>
       <sz val="16"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="15"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -480,14 +459,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FFFF4000"/>
+        <fgColor rgb="FF00A933"/>
+        <bgColor rgb="FF18A303"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00A933"/>
-        <bgColor rgb="FF18A303"/>
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FFFF4000"/>
       </patternFill>
     </fill>
     <fill>
@@ -801,6 +780,15 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
@@ -817,15 +805,6 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
@@ -878,11 +857,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -890,10 +873,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -906,7 +885,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -922,7 +901,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -974,7 +953,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -982,95 +961,95 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="24" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="25" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="24" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="24" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="25" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="15" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="15" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="16" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="18" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="28" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="16" xfId="28" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="28" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="28" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="18" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="13" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="19" xfId="24" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="28" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="13" xfId="28" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="28" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="28" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="19" xfId="27" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="20" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="21" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="21" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="22" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="20" xfId="26" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="21" xfId="26" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="21" xfId="26" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="22" xfId="26" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1078,171 +1057,171 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="23" xfId="21" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="24" xfId="21" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="21" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="21" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="23" xfId="24" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="24" xfId="24" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="24" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="24" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="15" xfId="20" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="15" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="16" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="18" xfId="20" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="16" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="18" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="25" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="26" xfId="20" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="25" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="26" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="13" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="27" xfId="24" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="13" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="27" xfId="27" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="28" xfId="24" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="28" xfId="27" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="20" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="21" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="21" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="22" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="21" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="19" xfId="24" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="20" xfId="26" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="21" xfId="26" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="21" xfId="26" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="22" xfId="26" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="24" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="19" xfId="27" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="29" xfId="21" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="30" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="29" xfId="24" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="30" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="31" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="32" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="33" xfId="25" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="28" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="31" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="32" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="33" xfId="28" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="28" xfId="26" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1258,55 +1237,55 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="35" xfId="21" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="36" xfId="21" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="21" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="35" xfId="24" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="36" xfId="24" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="24" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="24" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="27" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="24" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="27" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="20" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="37" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="20" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="37" xfId="26" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="24" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="27" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="32" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="23" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="32" xfId="26" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="26" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1318,15 +1297,15 @@
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Pivot Table Category" xfId="20"/>
-    <cellStyle name="Pivot Table Corner" xfId="21"/>
-    <cellStyle name="Pivot Table Field" xfId="22"/>
-    <cellStyle name="Pivot Table Result" xfId="23"/>
-    <cellStyle name="Pivot Table Title" xfId="24"/>
-    <cellStyle name="Pivot Table Value" xfId="25"/>
-    <cellStyle name="Heatmap" xfId="26"/>
-    <cellStyle name="Green Background" xfId="27"/>
-    <cellStyle name="Green" xfId="28"/>
+    <cellStyle name="Green" xfId="20"/>
+    <cellStyle name="Green Background" xfId="21"/>
+    <cellStyle name="Heatmap" xfId="22"/>
+    <cellStyle name="Pivot Table Category" xfId="23"/>
+    <cellStyle name="Pivot Table Corner" xfId="24"/>
+    <cellStyle name="Pivot Table Field" xfId="25"/>
+    <cellStyle name="Pivot Table Result" xfId="26"/>
+    <cellStyle name="Pivot Table Title" xfId="27"/>
+    <cellStyle name="Pivot Table Value" xfId="28"/>
   </cellStyles>
   <colors>
     <indexedColors>
@@ -1616,11 +1595,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="91026737"/>
-        <c:axId val="71725314"/>
+        <c:axId val="38430050"/>
+        <c:axId val="8672538"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="91026737"/>
+        <c:axId val="38430050"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1653,7 +1632,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71725314"/>
+        <c:crossAx val="8672538"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1661,7 +1640,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="71725314"/>
+        <c:axId val="8672538"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1703,7 +1682,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91026737"/>
+        <c:crossAx val="38430050"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1991,8 +1970,8 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="73254002"/>
-        <c:axId val="59847522"/>
+        <c:axId val="9126412"/>
+        <c:axId val="3164351"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2105,11 +2084,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="27372297"/>
-        <c:axId val="46153650"/>
+        <c:axId val="23082449"/>
+        <c:axId val="8684363"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="73254002"/>
+        <c:axId val="9126412"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2142,7 +2121,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59847522"/>
+        <c:crossAx val="3164351"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2150,7 +2129,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="59847522"/>
+        <c:axId val="3164351"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2192,12 +2171,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73254002"/>
+        <c:crossAx val="9126412"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="27372297"/>
+        <c:axId val="23082449"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2230,14 +2209,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46153650"/>
+        <c:crossAx val="8684363"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="46153650"/>
+        <c:axId val="8684363"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2270,7 +2249,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27372297"/>
+        <c:crossAx val="23082449"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2342,8 +2321,12 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1600" b="1" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>2022 net_sales: Pacific Crash</a:t>
             </a:r>
@@ -2408,12 +2391,17 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
@@ -2427,12 +2415,17 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -2493,8 +2486,8 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="4562748"/>
-        <c:axId val="58567975"/>
+        <c:axId val="13764844"/>
+        <c:axId val="32061920"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2535,8 +2528,12 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
@@ -2609,17 +2606,17 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="62710009"/>
-        <c:axId val="36035936"/>
+        <c:axId val="77335461"/>
+        <c:axId val="8856587"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="4562748"/>
+        <c:axId val="13764844"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2636,13 +2633,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58567975"/>
+        <c:crossAx val="32061920"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2650,7 +2651,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="58567975"/>
+        <c:axId val="32061920"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2665,7 +2666,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2682,18 +2683,22 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4562748"/>
+        <c:crossAx val="13764844"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="62710009"/>
+        <c:axId val="77335461"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2716,26 +2721,30 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36035936"/>
+        <c:crossAx val="8856587"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="36035936"/>
+        <c:axId val="8856587"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="r"/>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="none"/>
@@ -2752,13 +2761,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62710009"/>
+        <c:crossAx val="77335461"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2786,8 +2799,12 @@
         <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
               <a:uFillTx/>
               <a:latin typeface="Arial"/>
+              <a:ea typeface="DejaVu Sans"/>
             </a:defRPr>
           </a:pPr>
         </a:p>
@@ -2826,8 +2843,12 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1500" b="1" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>Margin Slight Drop</a:t>
             </a:r>
@@ -2888,6 +2909,7 @@
                     </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
@@ -2987,17 +3009,17 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="6928681"/>
-        <c:axId val="20518916"/>
+        <c:axId val="7631693"/>
+        <c:axId val="78201029"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="6928681"/>
+        <c:axId val="7631693"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3014,13 +3036,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20518916"/>
+        <c:crossAx val="78201029"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3028,13 +3054,13 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="20518916"/>
+        <c:axId val="78201029"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:numFmt formatCode="0.00%" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00%" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="none"/>
@@ -3051,13 +3077,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6928681"/>
+        <c:crossAx val="7631693"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3085,8 +3115,12 @@
         <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
               <a:uFillTx/>
               <a:latin typeface="Arial"/>
+              <a:ea typeface="DejaVu Sans"/>
             </a:defRPr>
           </a:pPr>
         </a:p>
@@ -3117,9 +3151,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>807840</xdr:colOff>
+      <xdr:colOff>807480</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>150120</xdr:rowOff>
+      <xdr:rowOff>149760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3128,7 +3162,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="5817240" y="352800"/>
-        <a:ext cx="5628600" cy="3165840"/>
+        <a:ext cx="5628240" cy="3165480"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3147,9 +3181,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1796760</xdr:colOff>
+      <xdr:colOff>1796400</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>73440</xdr:rowOff>
+      <xdr:rowOff>73080</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3158,7 +3192,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="52560" y="415800"/>
-        <a:ext cx="5669280" cy="3188880"/>
+        <a:ext cx="5668920" cy="3188520"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3177,9 +3211,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1834560</xdr:colOff>
+      <xdr:colOff>1834200</xdr:colOff>
       <xdr:row>46</xdr:row>
-      <xdr:rowOff>48960</xdr:rowOff>
+      <xdr:rowOff>48600</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3188,7 +3222,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="4574880"/>
-        <a:ext cx="5759640" cy="3239640"/>
+        <a:ext cx="5759280" cy="3239280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3207,9 +3241,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>130320</xdr:colOff>
+      <xdr:colOff>129960</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>137880</xdr:rowOff>
+      <xdr:rowOff>137520</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3218,7 +3252,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="5823360" y="3686400"/>
-        <a:ext cx="5757840" cy="3241440"/>
+        <a:ext cx="5757480" cy="3241080"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -4117,120 +4151,126 @@
       <c r="A3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="5" t="str">
+        <f aca="false">HYPERLINK("#01_Top3_Decliners!A1","01_top3_decliners")</f>
+        <v>01_top3_decliners</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>10</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="8" t="str">
+        <f aca="false">HYPERLINK("#02_Pacific_Crisis!A1","02_Pacific_Crisis")</f>
+        <v>02_Pacific_Crisis</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="E4" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>15</v>
-      </c>
       <c r="F4" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="8" t="str">
+        <f aca="false">HYPERLINK("#03_YoY_Negative!A1","03_YoY_Negative")</f>
+        <v>03_YoY_Negative</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="F5" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>21</v>
+      <c r="B6" s="8" t="str">
+        <f aca="false">HYPERLINK("#04_Bikes_Drivers!A1","04_Bikes_Drivers")</f>
+        <v>04_Bikes_Drivers</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>25</v>
+      <c r="B7" s="8" t="str">
+        <f aca="false">HYPERLINK("#05_High_Returns!A1","05_High_Returns")</f>
+        <v>05_High_Returns</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="11" t="s">
-        <v>29</v>
+      <c r="B8" s="11" t="str">
+        <f aca="false">HYPERLINK("#06_Top2_2022_Fix!A1","06_Top2_2022_Fix")</f>
+        <v>06_Top2_2022_Fix</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -4262,26 +4302,26 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B2" s="61" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B4" s="61" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4293,7 +4333,7 @@
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="107"/>
       <c r="B6" s="64" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C6" s="108"/>
       <c r="D6" s="63"/>
@@ -4301,24 +4341,24 @@
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="109"/>
       <c r="B7" s="110" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C7" s="111" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D7" s="112" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="68" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B8" s="70" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C8" s="70" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="D8" s="113"/>
     </row>
@@ -4352,7 +4392,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="117" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B11" s="118" t="n">
         <v>249.986760464594</v>
@@ -4393,33 +4433,33 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B2" s="61" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B4" s="61" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="62"/>
       <c r="B6" s="63"/>
       <c r="C6" s="64" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="D6" s="65"/>
       <c r="E6" s="65"/>
@@ -4427,22 +4467,22 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="67" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B7" s="68" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C7" s="69" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="D7" s="70" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="70" t="s">
+        <v>83</v>
+      </c>
+      <c r="F7" s="71" t="s">
         <v>86</v>
-      </c>
-      <c r="E7" s="70" t="s">
-        <v>89</v>
-      </c>
-      <c r="F7" s="71" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4450,7 +4490,7 @@
         <v>2022</v>
       </c>
       <c r="B8" s="73" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C8" s="74" t="n">
         <v>5689</v>
@@ -4468,7 +4508,7 @@
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="84"/>
       <c r="B9" s="85" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C9" s="86" t="n">
         <v>7132</v>
@@ -4485,7 +4525,7 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="90" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B10" s="91"/>
       <c r="C10" s="92" t="n">
@@ -4520,15 +4560,15 @@
   <dimension ref="A1:L49"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="19.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="19.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26.05"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="12"/>
       <c r="C1" s="13" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D1" s="13"/>
       <c r="E1" s="13"/>
@@ -4536,295 +4576,295 @@
       <c r="G1" s="13"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12"/>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="12"/>
-      <c r="K4" s="12"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="14"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
+      <c r="A5" s="14"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
+      <c r="A6" s="14"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
+      <c r="A7" s="14"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
+      <c r="A9" s="14"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="14"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="14"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
+      <c r="A11" s="14"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="14"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12"/>
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="14"/>
+      <c r="K12" s="14"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
+      <c r="A13" s="14"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="14"/>
+      <c r="K13" s="14"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
+      <c r="A14" s="14"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="14"/>
+      <c r="K14" s="14"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="14"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="12"/>
+      <c r="A16" s="14"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="12"/>
+      <c r="A17" s="14"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="14"/>
+      <c r="K17" s="14"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
+      <c r="A18" s="14"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
+      <c r="A19" s="14"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="14"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
+      <c r="A20" s="14"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="14"/>
+      <c r="K20" s="14"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="12"/>
-      <c r="I21" s="12"/>
-      <c r="J21" s="12"/>
-      <c r="K21" s="12"/>
+      <c r="A21" s="14"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="14"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="12"/>
-      <c r="I22" s="12"/>
-      <c r="J22" s="12"/>
-      <c r="K22" s="12"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14"/>
     </row>
     <row r="23" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>37</v>
+      <c r="A23" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>31</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="12"/>
-      <c r="I23" s="12"/>
-      <c r="J23" s="12"/>
-      <c r="K23" s="12"/>
-      <c r="L23" s="12"/>
+        <v>32</v>
+      </c>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="14"/>
+      <c r="K23" s="14"/>
+      <c r="L23" s="14"/>
     </row>
     <row r="24" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="16" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B24" s="17" t="n">
         <v>3218911</v>
@@ -4833,18 +4873,18 @@
         <v>215.7</v>
       </c>
       <c r="D24" s="19"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="12"/>
-      <c r="I24" s="12"/>
-      <c r="J24" s="12"/>
-      <c r="K24" s="12"/>
-      <c r="L24" s="12"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="14"/>
+      <c r="L24" s="14"/>
     </row>
     <row r="25" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B25" s="17" t="n">
         <v>3293497</v>
@@ -4853,18 +4893,18 @@
         <v>175.67</v>
       </c>
       <c r="D25" s="19"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="12"/>
-      <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
-      <c r="L25" s="12"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="14"/>
+      <c r="K25" s="14"/>
+      <c r="L25" s="14"/>
     </row>
     <row r="26" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B26" s="21" t="n">
         <v>34931</v>
@@ -4873,280 +4913,280 @@
         <v>253.81</v>
       </c>
       <c r="D26" s="23"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="12"/>
-      <c r="I26" s="12"/>
-      <c r="J26" s="12"/>
-      <c r="K26" s="12"/>
-      <c r="L26" s="12"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="14"/>
+      <c r="J26" s="14"/>
+      <c r="K26" s="14"/>
+      <c r="L26" s="14"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="12"/>
-      <c r="I27" s="12"/>
-      <c r="J27" s="12"/>
-      <c r="K27" s="12"/>
-      <c r="L27" s="12"/>
+      <c r="A27" s="14"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
+      <c r="I27" s="14"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="14"/>
+      <c r="L27" s="14"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="12"/>
-      <c r="G28" s="12"/>
-      <c r="H28" s="12"/>
-      <c r="I28" s="12"/>
-      <c r="J28" s="12"/>
-      <c r="K28" s="12"/>
-      <c r="L28" s="12"/>
+      <c r="A28" s="14"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="14"/>
+      <c r="J28" s="14"/>
+      <c r="K28" s="14"/>
+      <c r="L28" s="14"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="12"/>
-      <c r="I29" s="12"/>
-      <c r="J29" s="12"/>
-      <c r="K29" s="12"/>
-      <c r="L29" s="12"/>
+      <c r="A29" s="14"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="14"/>
+      <c r="H29" s="14"/>
+      <c r="I29" s="14"/>
+      <c r="J29" s="14"/>
+      <c r="K29" s="14"/>
+      <c r="L29" s="14"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="12"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="12"/>
-      <c r="I30" s="12"/>
-      <c r="J30" s="12"/>
-      <c r="K30" s="12"/>
-      <c r="L30" s="12"/>
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
+      <c r="I30" s="14"/>
+      <c r="J30" s="14"/>
+      <c r="K30" s="14"/>
+      <c r="L30" s="14"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="12"/>
-      <c r="I31" s="12"/>
-      <c r="J31" s="12"/>
-      <c r="K31" s="12"/>
-      <c r="L31" s="12"/>
+      <c r="A31" s="14"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="14"/>
+      <c r="J31" s="14"/>
+      <c r="K31" s="14"/>
+      <c r="L31" s="14"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="12"/>
-      <c r="B32" s="12"/>
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="12"/>
-      <c r="G32" s="12"/>
-      <c r="H32" s="12"/>
-      <c r="I32" s="12"/>
-      <c r="J32" s="12"/>
-      <c r="K32" s="12"/>
-      <c r="L32" s="12"/>
+      <c r="A32" s="14"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14"/>
+      <c r="I32" s="14"/>
+      <c r="J32" s="14"/>
+      <c r="K32" s="14"/>
+      <c r="L32" s="14"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="12"/>
-      <c r="B33" s="12"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="12"/>
-      <c r="I33" s="12"/>
-      <c r="J33" s="12"/>
-      <c r="K33" s="12"/>
-      <c r="L33" s="12"/>
+      <c r="A33" s="14"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
+      <c r="I33" s="14"/>
+      <c r="J33" s="14"/>
+      <c r="K33" s="14"/>
+      <c r="L33" s="14"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="12"/>
-      <c r="B34" s="12"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="12"/>
-      <c r="I34" s="12"/>
-      <c r="J34" s="12"/>
-      <c r="K34" s="12"/>
-      <c r="L34" s="12"/>
+      <c r="A34" s="14"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+      <c r="I34" s="14"/>
+      <c r="J34" s="14"/>
+      <c r="K34" s="14"/>
+      <c r="L34" s="14"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="12"/>
-      <c r="B35" s="12"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="12"/>
-      <c r="E35" s="12"/>
-      <c r="F35" s="12"/>
-      <c r="G35" s="12"/>
-      <c r="H35" s="12"/>
-      <c r="I35" s="12"/>
-      <c r="J35" s="12"/>
-      <c r="K35" s="12"/>
-      <c r="L35" s="12"/>
+      <c r="A35" s="14"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="14"/>
+      <c r="I35" s="14"/>
+      <c r="J35" s="14"/>
+      <c r="K35" s="14"/>
+      <c r="L35" s="14"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="12"/>
-      <c r="B36" s="12"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
-      <c r="G36" s="12"/>
-      <c r="H36" s="12"/>
-      <c r="I36" s="12"/>
-      <c r="J36" s="12"/>
-      <c r="K36" s="12"/>
-      <c r="L36" s="12"/>
+      <c r="A36" s="14"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="14"/>
+      <c r="I36" s="14"/>
+      <c r="J36" s="14"/>
+      <c r="K36" s="14"/>
+      <c r="L36" s="14"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="12"/>
-      <c r="B37" s="12"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="12"/>
-      <c r="F37" s="12"/>
-      <c r="G37" s="12"/>
-      <c r="H37" s="12"/>
-      <c r="I37" s="12"/>
-      <c r="J37" s="12"/>
-      <c r="K37" s="12"/>
-      <c r="L37" s="12"/>
+      <c r="A37" s="14"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="14"/>
+      <c r="H37" s="14"/>
+      <c r="I37" s="14"/>
+      <c r="J37" s="14"/>
+      <c r="K37" s="14"/>
+      <c r="L37" s="14"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12"/>
-      <c r="B38" s="12"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
-      <c r="F38" s="12"/>
-      <c r="G38" s="12"/>
-      <c r="H38" s="12"/>
-      <c r="I38" s="12"/>
-      <c r="J38" s="12"/>
-      <c r="K38" s="12"/>
-      <c r="L38" s="12"/>
+      <c r="A38" s="14"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14"/>
+      <c r="I38" s="14"/>
+      <c r="J38" s="14"/>
+      <c r="K38" s="14"/>
+      <c r="L38" s="14"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="12"/>
-      <c r="B39" s="12"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="12"/>
-      <c r="F39" s="12"/>
-      <c r="G39" s="12"/>
-      <c r="H39" s="12"/>
-      <c r="I39" s="12"/>
-      <c r="J39" s="12"/>
-      <c r="K39" s="12"/>
-      <c r="L39" s="12"/>
+      <c r="A39" s="14"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="14"/>
+      <c r="H39" s="14"/>
+      <c r="I39" s="14"/>
+      <c r="J39" s="14"/>
+      <c r="K39" s="14"/>
+      <c r="L39" s="14"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="12"/>
-      <c r="B40" s="12"/>
-      <c r="C40" s="12"/>
-      <c r="D40" s="12"/>
-      <c r="E40" s="12"/>
-      <c r="F40" s="12"/>
-      <c r="G40" s="12"/>
-      <c r="H40" s="12"/>
-      <c r="I40" s="12"/>
-      <c r="J40" s="12"/>
-      <c r="K40" s="12"/>
-      <c r="L40" s="12"/>
+      <c r="A40" s="14"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="14"/>
+      <c r="H40" s="14"/>
+      <c r="I40" s="14"/>
+      <c r="J40" s="14"/>
+      <c r="K40" s="14"/>
+      <c r="L40" s="14"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="12"/>
-      <c r="B41" s="12"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="12"/>
-      <c r="E41" s="12"/>
-      <c r="F41" s="12"/>
-      <c r="G41" s="12"/>
-      <c r="H41" s="12"/>
-      <c r="I41" s="12"/>
-      <c r="J41" s="12"/>
-      <c r="K41" s="12"/>
-      <c r="L41" s="12"/>
+      <c r="A41" s="14"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="14"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="14"/>
+      <c r="G41" s="14"/>
+      <c r="H41" s="14"/>
+      <c r="I41" s="14"/>
+      <c r="J41" s="14"/>
+      <c r="K41" s="14"/>
+      <c r="L41" s="14"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="12"/>
-      <c r="B42" s="12"/>
-      <c r="C42" s="12"/>
-      <c r="D42" s="12"/>
-      <c r="E42" s="12"/>
-      <c r="F42" s="12"/>
-      <c r="G42" s="12"/>
-      <c r="H42" s="12"/>
-      <c r="I42" s="12"/>
-      <c r="J42" s="12"/>
-      <c r="K42" s="12"/>
-      <c r="L42" s="12"/>
+      <c r="A42" s="14"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
+      <c r="G42" s="14"/>
+      <c r="H42" s="14"/>
+      <c r="I42" s="14"/>
+      <c r="J42" s="14"/>
+      <c r="K42" s="14"/>
+      <c r="L42" s="14"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="12"/>
-      <c r="B43" s="12"/>
-      <c r="C43" s="12"/>
-      <c r="D43" s="12"/>
+      <c r="A43" s="14"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="12"/>
-      <c r="B44" s="12"/>
-      <c r="C44" s="12"/>
-      <c r="D44" s="12"/>
+      <c r="A44" s="14"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="14"/>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="12"/>
-      <c r="B45" s="12"/>
-      <c r="C45" s="12"/>
-      <c r="D45" s="12"/>
+      <c r="A45" s="14"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="12"/>
-      <c r="B46" s="12"/>
-      <c r="C46" s="12"/>
-      <c r="D46" s="12"/>
+      <c r="A46" s="14"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="14"/>
+      <c r="D46" s="14"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="12"/>
-      <c r="B47" s="12"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="12"/>
+      <c r="A47" s="14"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="12"/>
-      <c r="B48" s="12"/>
-      <c r="C48" s="12"/>
-      <c r="D48" s="12"/>
+      <c r="A48" s="14"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="14"/>
+      <c r="D48" s="14"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="12"/>
-      <c r="B49" s="12"/>
-      <c r="C49" s="12"/>
-      <c r="D49" s="12"/>
+      <c r="A49" s="14"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="14"/>
+      <c r="D49" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -5172,7 +5212,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.12"/>
@@ -5183,12 +5223,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="13.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="14.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="20.07"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B1" s="24" t="n">
         <v>2021</v>
@@ -5197,33 +5237,33 @@
         <v>2022</v>
       </c>
       <c r="D1" s="24" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="E1" s="24" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="G1" s="24" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="H1" s="24" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="I1" s="24" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="J1" s="24" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="K1" s="24" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="25" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B2" s="25" t="n">
         <v>36230</v>
@@ -5238,7 +5278,7 @@
         <v>0.2507</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="G2" s="26" t="n">
         <v>67888</v>
@@ -5247,7 +5287,7 @@
         <v>3</v>
       </c>
       <c r="I2" s="28" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="J2" s="29" t="n">
         <v>3218911</v>
@@ -5258,7 +5298,7 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="25" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="B3" s="25" t="n">
         <v>3690735</v>
@@ -5273,7 +5313,7 @@
         <v>-0.0214</v>
       </c>
       <c r="F3" s="25" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="G3" s="26" t="n">
         <v>-169476</v>
@@ -5282,7 +5322,7 @@
         <v>1</v>
       </c>
       <c r="I3" s="28" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="J3" s="29" t="n">
         <v>3293497</v>
@@ -5293,7 +5333,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="25" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="B4" s="27" t="n">
         <v>0.4255</v>
@@ -5308,7 +5348,7 @@
         <v>-0.0049</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="G4" s="26" t="n">
         <v>23533</v>
@@ -5317,7 +5357,7 @@
         <v>2</v>
       </c>
       <c r="I4" s="28" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="J4" s="29" t="n">
         <v>34931</v>
@@ -5325,26 +5365,6 @@
       <c r="K4" s="30" t="n">
         <v>253.81</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I11" s="0"/>
-      <c r="J11" s="0"/>
-      <c r="K11" s="0"/>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I12" s="0"/>
-      <c r="J12" s="0"/>
-      <c r="K12" s="0"/>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I13" s="0"/>
-      <c r="J13" s="0"/>
-      <c r="K13" s="0"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I14" s="0"/>
-      <c r="J14" s="0"/>
-      <c r="K14" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -5381,82 +5401,82 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="33" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="33" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="H1" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="I1" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="D1" s="34" t="s">
+      <c r="J1" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="34" t="s">
+      <c r="K1" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="F1" s="34" t="s">
+      <c r="L1" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="G1" s="34" t="s">
+      <c r="M1" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="H1" s="34" t="s">
+      <c r="N1" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="I1" s="34" t="s">
+      <c r="O1" s="35" t="s">
         <v>62</v>
       </c>
-      <c r="J1" s="34" t="s">
+      <c r="P1" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="K1" s="34" t="s">
+      <c r="Q1" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="L1" s="34" t="s">
+      <c r="R1" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="M1" s="34" t="s">
+      <c r="S1" s="35" t="s">
         <v>66</v>
       </c>
-      <c r="N1" s="34" t="s">
+      <c r="T1" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="O1" s="35" t="s">
+      <c r="U1" s="35" t="s">
         <v>68</v>
       </c>
-      <c r="P1" s="35" t="s">
+      <c r="V1" s="35" t="s">
         <v>69</v>
       </c>
-      <c r="Q1" s="35" t="s">
+      <c r="W1" s="35" t="s">
         <v>70</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="X1" s="35" t="s">
         <v>71</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="Y1" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z1" s="35" t="s">
         <v>72</v>
-      </c>
-      <c r="T1" s="35" t="s">
-        <v>73</v>
-      </c>
-      <c r="U1" s="35" t="s">
-        <v>74</v>
-      </c>
-      <c r="V1" s="35" t="s">
-        <v>75</v>
-      </c>
-      <c r="W1" s="35" t="s">
-        <v>76</v>
-      </c>
-      <c r="X1" s="35" t="s">
-        <v>77</v>
-      </c>
-      <c r="Y1" s="35" t="s">
-        <v>37</v>
-      </c>
-      <c r="Z1" s="35" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5503,7 +5523,7 @@
         <v>42.55</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="P2" s="1" t="n">
         <v>0</v>
@@ -5524,7 +5544,7 @@
         <v>0</v>
       </c>
       <c r="V2" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="W2" s="1" t="n">
         <v>0</v>
@@ -5536,7 +5556,7 @@
         <v>0</v>
       </c>
       <c r="Z2" s="1" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5583,7 +5603,7 @@
         <v>42.34</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="P3" s="1" t="n">
         <v>0</v>
@@ -5604,7 +5624,7 @@
         <v>0</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="W3" s="1" t="n">
         <v>0</v>
@@ -5616,7 +5636,7 @@
         <v>0</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5663,7 +5683,7 @@
         <v>0</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="P4" s="1" t="n">
         <v>399342.117799956</v>
@@ -5684,7 +5704,7 @@
         <v>6</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="W4" s="1" t="n">
         <v>0</v>
@@ -5696,7 +5716,7 @@
         <v>0</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5743,7 +5763,7 @@
         <v>0</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="P5" s="1" t="n">
         <v>507330.989199908</v>
@@ -5764,7 +5784,7 @@
         <v>3</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="W5" s="1" t="n">
         <v>0</v>
@@ -5776,7 +5796,7 @@
         <v>0</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5823,7 +5843,7 @@
         <v>0</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="P6" s="1" t="n">
         <v>8768706.98490015</v>
@@ -5844,7 +5864,7 @@
         <v>4</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="W6" s="1" t="n">
         <v>0</v>
@@ -5856,7 +5876,7 @@
         <v>0</v>
       </c>
       <c r="Z6" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5903,7 +5923,7 @@
         <v>0</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="P7" s="1" t="n">
         <v>8468854.53000019</v>
@@ -5924,7 +5944,7 @@
         <v>1</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="W7" s="1" t="n">
         <v>0</v>
@@ -5936,7 +5956,7 @@
         <v>0</v>
       </c>
       <c r="Z7" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5983,7 +6003,7 @@
         <v>0</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="P8" s="1" t="n">
         <v>156154.688999999</v>
@@ -6004,7 +6024,7 @@
         <v>5</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="W8" s="1" t="n">
         <v>0</v>
@@ -6016,7 +6036,7 @@
         <v>0</v>
       </c>
       <c r="Z8" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6063,7 +6083,7 @@
         <v>0</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="P9" s="1" t="n">
         <v>209263.928099994</v>
@@ -6084,7 +6104,7 @@
         <v>2</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="W9" s="1" t="n">
         <v>0</v>
@@ -6096,7 +6116,7 @@
         <v>0</v>
       </c>
       <c r="Z9" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6143,7 +6163,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="P10" s="1" t="n">
         <v>0</v>
@@ -6164,7 +6184,7 @@
         <v>0</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="W10" s="1" t="n">
         <v>864233</v>
@@ -6176,7 +6196,7 @@
         <v>284.275128347168</v>
       </c>
       <c r="Z10" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6223,7 +6243,7 @@
         <v>0</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="P11" s="1" t="n">
         <v>0</v>
@@ -6244,7 +6264,7 @@
         <v>0</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="W11" s="1" t="n">
         <v>2218218</v>
@@ -6256,7 +6276,7 @@
         <v>190.12575110637</v>
       </c>
       <c r="Z11" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6303,7 +6323,7 @@
         <v>0</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="P12" s="1" t="n">
         <v>0</v>
@@ -6324,7 +6344,7 @@
         <v>0</v>
       </c>
       <c r="V12" s="1" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="W12" s="1" t="n">
         <v>1249024</v>
@@ -6336,7 +6356,7 @@
         <v>375.741416680663</v>
       </c>
       <c r="Z12" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6383,7 +6403,7 @@
         <v>0</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="P13" s="1" t="n">
         <v>0</v>
@@ -6404,7 +6424,7 @@
         <v>0</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="W13" s="1" t="n">
         <v>1353420</v>
@@ -6416,7 +6436,7 @@
         <v>215.69839258202</v>
       </c>
       <c r="Z13" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6463,7 +6483,7 @@
         <v>0</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="P14" s="1" t="n">
         <v>0</v>
@@ -6484,7 +6504,7 @@
         <v>0</v>
       </c>
       <c r="V14" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="W14" s="1" t="n">
         <v>3496046</v>
@@ -6496,7 +6516,7 @@
         <v>175.669374322156</v>
       </c>
       <c r="Z14" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6543,7 +6563,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="P15" s="1" t="n">
         <v>0</v>
@@ -6564,7 +6584,7 @@
         <v>0</v>
       </c>
       <c r="V15" s="1" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="W15" s="1" t="n">
         <v>1944835</v>
@@ -6576,7 +6596,7 @@
         <v>253.814111575181</v>
       </c>
       <c r="Z15" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6645,10 +6665,10 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="36" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B2" s="37" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C2" s="0"/>
       <c r="D2" s="0"/>
@@ -6661,10 +6681,10 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="36" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C3" s="0"/>
       <c r="D3" s="0"/>
@@ -6677,10 +6697,10 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="36" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C4" s="0"/>
       <c r="D4" s="0"/>
@@ -6706,7 +6726,7 @@
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="38"/>
       <c r="B6" s="39" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C6" s="40"/>
       <c r="D6" s="40"/>
@@ -6719,34 +6739,34 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="42" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B7" s="43" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="44" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="44" t="s">
+        <v>81</v>
+      </c>
+      <c r="E7" s="44" t="s">
+        <v>82</v>
+      </c>
+      <c r="F7" s="44" t="s">
+        <v>83</v>
+      </c>
+      <c r="G7" s="44" t="s">
+        <v>84</v>
+      </c>
+      <c r="H7" s="44" t="s">
+        <v>82</v>
+      </c>
+      <c r="I7" s="44" t="s">
         <v>85</v>
       </c>
-      <c r="C7" s="44" t="s">
+      <c r="J7" s="45" t="s">
         <v>86</v>
-      </c>
-      <c r="D7" s="44" t="s">
-        <v>87</v>
-      </c>
-      <c r="E7" s="44" t="s">
-        <v>88</v>
-      </c>
-      <c r="F7" s="44" t="s">
-        <v>89</v>
-      </c>
-      <c r="G7" s="44" t="s">
-        <v>90</v>
-      </c>
-      <c r="H7" s="44" t="s">
-        <v>88</v>
-      </c>
-      <c r="I7" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="J7" s="45" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6815,7 +6835,7 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="56" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B10" s="57" t="n">
         <v>163088</v>
@@ -6874,33 +6894,33 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B2" s="61" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B4" s="61" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="62"/>
       <c r="B6" s="63"/>
       <c r="C6" s="64" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="D6" s="65"/>
       <c r="E6" s="65"/>
@@ -6908,22 +6928,22 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="67" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B7" s="68" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C7" s="69" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="D7" s="70" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="70" t="s">
+        <v>83</v>
+      </c>
+      <c r="F7" s="71" t="s">
         <v>86</v>
-      </c>
-      <c r="E7" s="70" t="s">
-        <v>89</v>
-      </c>
-      <c r="F7" s="71" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6931,7 +6951,7 @@
         <v>2022</v>
       </c>
       <c r="B8" s="73" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C8" s="74" t="n">
         <v>32493</v>
@@ -6949,7 +6969,7 @@
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="78"/>
       <c r="B9" s="79" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C9" s="80" t="n">
         <v>5689</v>
@@ -6967,7 +6987,7 @@
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="84"/>
       <c r="B10" s="85" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C10" s="86" t="n">
         <v>7132</v>
@@ -6984,7 +7004,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="90" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B11" s="91"/>
       <c r="C11" s="92" t="n">
@@ -7026,26 +7046,26 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B2" s="61" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B4" s="61" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7055,13 +7075,13 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="67" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B7" s="70" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C7" s="71" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7088,7 +7108,7 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="97" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B10" s="94" t="n">
         <v>314.777764127922</v>
@@ -7126,23 +7146,23 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B2" s="61" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B4" s="61" t="n">
         <v>-2.14</v>
@@ -7151,7 +7171,7 @@
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="96"/>
       <c r="B6" s="64" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C6" s="65"/>
       <c r="D6" s="65"/>
@@ -7161,25 +7181,25 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="67" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B7" s="69" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="70" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="70" t="s">
+        <v>81</v>
+      </c>
+      <c r="E7" s="70" t="s">
+        <v>82</v>
+      </c>
+      <c r="F7" s="70" t="s">
+        <v>82</v>
+      </c>
+      <c r="G7" s="99" t="s">
         <v>85</v>
-      </c>
-      <c r="C7" s="70" t="s">
-        <v>86</v>
-      </c>
-      <c r="D7" s="70" t="s">
-        <v>87</v>
-      </c>
-      <c r="E7" s="70" t="s">
-        <v>88</v>
-      </c>
-      <c r="F7" s="70" t="s">
-        <v>88</v>
-      </c>
-      <c r="G7" s="99" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7207,7 +7227,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="97" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B9" s="92" t="n">
         <v>45314</v>
@@ -7257,32 +7277,32 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B2" s="61" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B4" s="61" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="96"/>
       <c r="B6" s="64" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C6" s="65"/>
       <c r="D6" s="65"/>
@@ -7291,22 +7311,22 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="67" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B7" s="69" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C7" s="70" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="70" t="s">
+        <v>83</v>
+      </c>
+      <c r="E7" s="70" t="s">
         <v>86</v>
       </c>
-      <c r="D7" s="70" t="s">
-        <v>89</v>
-      </c>
-      <c r="E7" s="70" t="s">
-        <v>92</v>
-      </c>
       <c r="F7" s="71" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7351,7 +7371,7 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="97" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B10" s="92" t="n">
         <v>11299</v>

</xml_diff>